<commit_message>
chore: update master tracker 2026-08-28 23:54 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-28 23:35</t>
+          <t>2026-08-28 23:54</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -536,7 +536,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>47</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -570,19 +570,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="56" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -634,6 +634,582 @@
       <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Drive Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2018-12-23_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2018-12-23</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>biometria</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2018/labs/2018-12-23_labs_quest-mx_general.pdf</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2018/labs/2018-12-23_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1yXIoXfmo7MCVTJgg-7x67ocMMSYp8yJI/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2019-03-18_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2019-03-18</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>tiroideo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2019/labs/2019-03-18_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2019/labs/2019-03-18_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>no_change</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/12dTyXCSpbmK54M3uu1_8ONu0ffcKoXM_/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2019-03-22_labs_quest-mx_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2019-03-22</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>tiroglobulina</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2019/labs/2019-03-22_labs_quest-mx_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2019/labs/2019-03-22_labs_quest-mx_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>no_change</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1W-QWVHwJaEsG61mMJgBqRt6_Wz4yUciZ/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2019-05-15_labs_quest-mx_general-orina.pdf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2019-05-15</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>general-orina</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2019/labs/2019-05-15_labs_quest-mx_orina.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1HIIPFPUwJQdLc9Qi-rUbP-wOLn8SRXtA/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2019-09-13</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>tiroideo</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>no_change</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1txD2M8pAnAInDxjvL3pi712wRwmPTsPT/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2019-12-24_labs_quest-mx_perfil-lipidico.pdf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2019-12-24</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>perfil-lipidico</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2019/labs/2019-12-24_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2019/labs/2019-12-24_labs_quest-mx_perfil-lipidico.pdf</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1qiH2_frLbKJ2vF2j6ICW6j9SRmbxxGU0/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2020-04-17_labs_quest-mx_perfil-lipidico.pdf</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2020-04-17</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>perfil-lipidico</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2020/labs/2020-04-17_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2020/labs/2020-04-17_labs_quest-mx_perfil-lipidico.pdf</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1pdBluP-dzl_wE0f_FWKaNH-l1mFrxZvw/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2020-04-28_labs_quest-mx_perfil-lipidico.pdf</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2020-04-28</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>perfil-lipidico</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2020/labs/2020-04-28_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2020/labs/2020-04-28_labs_quest-mx_perfil-lipidico.pdf</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1JIAoEhyttwxc6Cv_SHEYfi9jodXjI9R7/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2020-05-25</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>perfil-tiroideo</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2020/labs/2020-05-25_labs_quest-mx_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1sNLAT_auII9ux0kE0dNzDNi-5cmWi4H_/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2020-06-15_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2020-06-15</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>tiroideo</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2020/labs/2020-06-15_labs_quest-mx_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2020/labs/2020-06-15_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1xq4z67ZNSeS-Ir5m3rtl17ElitnuZ2j4/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2021-12-22_labs_quest-mx_perfil-lipidico.pdf</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2021-12-22</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>perfil-lipidico</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2021/labs/2021-12-22_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2021/labs/2021-12-22_labs_quest-mx_perfil-lipidico.pdf</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1biQ7aNiS2p3mTi15rbgT2OE1HBr6scUP/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-17_labs_quest-mx_general.pdf</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026/labs/2026-04-17_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2026/labs/2026-04-17_labs_quest-mx_general.pdf</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1UFeodi51jpRW9wcmxggZwTnSBr6yz8Yn/view</t>
         </is>
       </c>
     </row>
@@ -726,19 +1302,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -790,6 +1366,54 @@
       <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Drive Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>hospital-angeles-lomas</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ultrasonido-tiroides</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonido_tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1M2fSSCUpWpLLZ_bJAAfgT1LckEtoI9gE/view</t>
         </is>
       </c>
     </row>
@@ -804,19 +1428,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="39" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -868,6 +1492,54 @@
       <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Drive Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-05-25_inbody_hospital-angeles-lomas_composicion-corporal.jpg</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>hospital-angeles-lomas</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>composicion-corporal</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026/inbody/2026-05-25_inbody_mnc.jpg</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026/inbody/2026-05-25_inbody_hospital-angeles-lomas_composicion-corporal.jpg</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1xsRRCzzETUWiVniCP37RdKGqnoAWf948/view</t>
         </is>
       </c>
     </row>
@@ -960,7 +1632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J48"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1030,7 +1702,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>REVISAR_2018-12-23_labs_quest-mx_general.pdf</t>
+          <t>REVISAR_2018-12-24_patologia_metastasis-papilar.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -1039,12 +1711,12 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2018/labs/2018-12-23_labs_quest-mx_general.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_metastasis-papilar.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2018-12-23_labs_quest-mx_general.pdf</t>
+          <t>_REVISAR/REVISAR_2018-12-24_patologia_metastasis-papilar.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1054,19 +1726,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 19927420 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW1yRyzE4Fj6TLDDRr6A'}</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1yXIoXfmo7MCVTJgg-7x67ocMMSYp8yJI/view</t>
+          <t>https://drive.google.com/file/d/17YnpChBP-Wq4Q3nCB9g5lk7n1STZAUcK/view</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>REVISAR_2018-12-24_patologia_metastasis-papilar.pdf</t>
+          <t>REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -1075,12 +1747,12 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_metastasis-papilar.pdf</t>
+          <t>2019/labs/2019-04-12_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2018-12-24_patologia_metastasis-papilar.pdf</t>
+          <t>_REVISAR/REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1090,19 +1762,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 17873820 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW1xi5amQ8Kc1kQ6K9xY'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17YnpChBP-Wq4Q3nCB9g5lk7n1STZAUcK/view</t>
+          <t>https://drive.google.com/file/d/10k9PIQTuP00FjD3--JFilIztJsAHzLex/view</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>REVISAR_2019-03-18_labs_quest-mx_tiroideo.pdf</t>
+          <t>REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -1111,12 +1783,12 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2019/labs/2019-03-18_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/labs/2019-06-02_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-03-18_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1126,19 +1798,19 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 14749848 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW21U2pjQWqUrd77Mm5T'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/12dTyXCSpbmK54M3uu1_8ONu0ffcKoXM_/view</t>
+          <t>https://drive.google.com/file/d/1ffwqecdhzalYlS6o1XRwtznJRSrJ-KGV/view</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REVISAR_2019-03-22_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -1147,12 +1819,12 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2019/labs/2019-03-22_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>2019/radiologia/2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-03-22_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>_REVISAR/REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1162,19 +1834,19 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 13457600 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW23UCoPoxBka2geRTa8'}</t>
+          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1W-QWVHwJaEsG61mMJgBqRt6_Wz4yUciZ/view</t>
+          <t>https://drive.google.com/file/d/17PCU-FXw71gWbY5q8Id6_YjqM-d_BoVz/view</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
+          <t>REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -1183,12 +1855,12 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2019/labs/2019-04-12_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/radiologia/2019-01-09_patologia_diseccion-cuello.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1198,19 +1870,19 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 15307956 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW1zeRNfH4gxgfihuv5X'}</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/10k9PIQTuP00FjD3--JFilIztJsAHzLex/view</t>
+          <t>https://drive.google.com/file/d/1LYjog3waD7Oso0nAvtdOUpNEqfwYTmgY/view</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>REVISAR_2019-05-15_labs_quest-mx_orina.pdf</t>
+          <t>REVISAR_2019-03-11_nuclear_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -1219,12 +1891,12 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_orina.pdf</t>
+          <t>2019/radiologia/2019-03-11_nuclear_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-05-15_labs_quest-mx_orina.pdf</t>
+          <t>_REVISAR/REVISAR_2019-03-11_nuclear_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1234,19 +1906,19 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 17158804 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW21zyut3E3okgzxeTR9'}</t>
+          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1HIIPFPUwJQdLc9Qi-rUbP-wOLn8SRXtA/view</t>
+          <t>https://drive.google.com/file/d/1aia7BfJ-fw8149Vg-5iKgJZJ7g2IHK8l/view</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
+          <t>REVISAR_2019-04-29_patologia_braf-v600e.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -1255,12 +1927,12 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2019/labs/2019-06-02_labs_quest-mx_general.pdf</t>
+          <t>2019/radiologia/2019-04-29_patologia_braf-v600e.pdf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
+          <t>_REVISAR/REVISAR_2019-04-29_patologia_braf-v600e.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1270,19 +1942,19 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 14920616 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW22YjdJ48Pn3TmqaGMh'}</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ffwqecdhzalYlS6o1XRwtznJRSrJ-KGV/view</t>
+          <t>https://drive.google.com/file/d/1J4gLdlbUkRGF_aKpx6xqt-qvIimskL5x/view</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>REVISAR_2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>REVISAR_2019-08-21_rx_torax.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -1291,12 +1963,12 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/radiologia/2019-08-21_rx_torax.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/REVISAR_2019-08-21_rx_torax.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1306,19 +1978,19 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 14257324 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2312B5RsJSFAtiJ7Wd'}</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1txD2M8pAnAInDxjvL3pi712wRwmPTsPT/view</t>
+          <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>REVISAR_2019-12-24_labs_quest-mx_tiroideo.pdf</t>
+          <t>REVISAR_2019-08-21_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -1327,12 +1999,12 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2019/labs/2019-12-24_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/ultrasonidos/2019-08-21_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-12-24_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/REVISAR_2019-08-21_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1342,19 +2014,19 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 404 - {'type': 'error', 'error': {'type': 'not_found_error', 'message': 'model: claude-sonnet-4-20250514'}, 'request_id': 'req_011CeW211Ph9iqn47E8rxZPz'}</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1qiH2_frLbKJ2vF2j6ICW6j9SRmbxxGU0/view</t>
+          <t>https://drive.google.com/file/d/10vh3Q4UHpBkOWSKLZAkMTumYwzVgfypN/view</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
+          <t>REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -1363,12 +2035,12 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2020/labs/2020-12-10_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
+          <t>_REVISAR/REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1378,19 +2050,19 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 19243660 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW24dCZVqhSPv97ncZ8G'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17PCU-FXw71gWbY5q8Id6_YjqM-d_BoVz/view</t>
+          <t>https://drive.google.com/file/d/1kkEH36xcggv0M0nYPQP1z7GX8a6d1Q-3/view</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
+          <t>REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -1399,12 +2071,12 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-01-09_patologia_diseccion-cuello.pdf</t>
+          <t>2020/radiologia/2020-06-01_patologia_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1414,19 +2086,19 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 25264556 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW25xUxSVL9UxVeh2v9i'}</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1LYjog3waD7Oso0nAvtdOUpNEqfwYTmgY/view</t>
+          <t>https://drive.google.com/file/d/19PXsFTn8Hf3QyTUKLZGk5MDFmI978hn4/view</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>REVISAR_2019-03-11_nuclear_rastreo-yodo.pdf</t>
+          <t>REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -1435,12 +2107,12 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-03-11_nuclear_rastreo-yodo.pdf</t>
+          <t>2020/radiologia/2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-03-11_nuclear_rastreo-yodo.pdf</t>
+          <t>_REVISAR/REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1450,19 +2122,19 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 17511668 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW26aCHzVauXCkPesZXs'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1aia7BfJ-fw8149Vg-5iKgJZJ7g2IHK8l/view</t>
+          <t>https://drive.google.com/file/d/1GcHOu5s7I3sn3A91BaqbSp0DkbtRu3tU/view</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>REVISAR_2019-04-29_patologia_braf-v600e.pdf</t>
+          <t>REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -1471,12 +2143,12 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-04-29_patologia_braf-v600e.pdf</t>
+          <t>2020/radiologia/2020-06-05_patologia_ganglios-cervicales.pdf</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-04-29_patologia_braf-v600e.pdf</t>
+          <t>_REVISAR/REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1486,19 +2158,19 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 16220412 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW25BCuUW3bBiqkwLE8N'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1J4gLdlbUkRGF_aKpx6xqt-qvIimskL5x/view</t>
+          <t>https://drive.google.com/file/d/1rRgSwtQWA6h02p8yGoUlgmc6Qc3x6DsU/view</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>REVISAR_2019-08-21_rx_torax.pdf</t>
+          <t>REVISAR_2020-07-14_nuclear_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -1507,12 +2179,12 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-08-21_rx_torax.pdf</t>
+          <t>2020/radiologia/2020-07-14_nuclear_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-08-21_rx_torax.pdf</t>
+          <t>_REVISAR/REVISAR_2020-07-14_nuclear_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1522,19 +2194,19 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 12541952 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW23zsGfk9RtcD43wY5R'}</t>
+          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
+          <t>https://drive.google.com/file/d/1rf96g6MjMv984xtt0QyWjjnklULtvj3N/view</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>REVISAR_2019-08-21_ultrasonido_cuello.pdf</t>
+          <t>REVISAR_2020-05-23_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -1543,12 +2215,12 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2019/ultrasonidos/2019-08-21_ultrasonido_cuello.pdf</t>
+          <t>2020/ultrasonidos/2020-05-23_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-08-21_ultrasonido_cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2020-05-23_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1558,19 +2230,19 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 18326828 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW1z57A16uAWYDiCWQC2'}</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/10vh3Q4UHpBkOWSKLZAkMTumYwzVgfypN/view</t>
+          <t>https://drive.google.com/file/d/1z424DznUpGdbjwRU0dlzICuxFdSfVYW1/view</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>REVISAR_2020-04-17_labs_quest-mx_tiroideo.pdf</t>
+          <t>REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -1579,12 +2251,12 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2020/labs/2020-04-17_labs_quest-mx_tiroideo.pdf</t>
+          <t>2021/labs/2021-06-07_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-04-17_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1594,19 +2266,19 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 15552692 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2CnzA1D4Zy6vqiqptd'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1pdBluP-dzl_wE0f_FWKaNH-l1mFrxZvw/view</t>
+          <t>https://drive.google.com/file/d/1CASli8xRI7Y1wLKR6oLBZ3JQRf-Y1KdU/view</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>REVISAR_2020-04-28_labs_quest-mx_tiroideo.pdf</t>
+          <t>REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -1615,12 +2287,12 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2020/labs/2020-04-28_labs_quest-mx_tiroideo.pdf</t>
+          <t>2021/labs/2021-06-07_labs_quest-mx_biometria_2.pdf</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-04-28_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1630,19 +2302,19 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 404 - {'type': 'error', 'error': {'type': 'not_found_error', 'message': 'model: claude-sonnet-4-20250514'}, 'request_id': 'req_011CeW2D85c6i1B8VeNG78KR'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1JIAoEhyttwxc6Cv_SHEYfi9jodXjI9R7/view</t>
+          <t>https://drive.google.com/file/d/1nuqeeVhX0deJ7BwXzsKAfsUsOPgi_HLF/view</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>REVISAR_2020-05-25_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>REVISAR_2021-12-22_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -1651,12 +2323,12 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>2021/ultrasonidos/2021-12-22_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-05-25_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>_REVISAR/REVISAR_2021-12-22_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1666,19 +2338,19 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 11508912 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2DVf8vKBepxn8GKYdS'}</t>
+          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1sNLAT_auII9ux0kE0dNzDNi-5cmWi4H_/view</t>
+          <t>https://drive.google.com/file/d/1SB7Z_2GOg3VG7gV0fVUUXPj0gYamdbXo/view</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>REVISAR_2020-06-15_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -1687,12 +2359,12 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2020/labs/2020-06-15_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>2022/labs/2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-06-15_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>_REVISAR/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1702,19 +2374,19 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 12707032 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2Dvb5SuavCKAzJD9PB'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1xq4z67ZNSeS-Ir5m3rtl17ElitnuZ2j4/view</t>
+          <t>https://drive.google.com/file/d/1UECfx-gSSTtlJVsvrEzkGi6uh5okeiN-/view</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
+          <t>REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -1723,12 +2395,12 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2020/labs/2020-12-10_labs_quest-mx_tiroideo.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1738,19 +2410,19 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 12889824 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2EN2HMvx8vzBnBoTYN'}</t>
+          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1kkEH36xcggv0M0nYPQP1z7GX8a6d1Q-3/view</t>
+          <t>https://drive.google.com/file/d/1yCWX0hgZnqKA57F22HZispDTzJKYOazt/view</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
+          <t>REVISAR_2022-06-06_ultrasonido_tiroides.pdf</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -1759,12 +2431,12 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2020/radiologia/2020-06-01_patologia_baaf-ganglio.pdf</t>
+          <t>2022/ultrasonidos/2022-06-06_ultrasonido_tiroides.pdf</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
+          <t>_REVISAR/REVISAR_2022-06-06_ultrasonido_tiroides.pdf</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1774,19 +2446,19 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 16069944 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2EuYMFt1j9FaDRMKJp'}</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/19PXsFTn8Hf3QyTUKLZGk5MDFmI978hn4/view</t>
+          <t>https://drive.google.com/file/d/1-rG8B2xpt-B6Okw5xi7AskcAYsnjOxiv/view</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
+          <t>REVISAR_2022-10-03_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -1795,12 +2467,12 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>2020/radiologia/2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2022/ultrasonidos/2022-10-03_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
+          <t>_REVISAR/REVISAR_2022-10-03_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1810,19 +2482,19 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 12717220 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2FRbcrdrn4kquawK5A'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1GcHOu5s7I3sn3A91BaqbSp0DkbtRu3tU/view</t>
+          <t>https://drive.google.com/file/d/11zttxbCEKhjP1KQWynf-lKor0LmoduHe/view</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
+          <t>REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -1831,12 +2503,12 @@
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>2020/radiologia/2020-06-05_patologia_ganglios-cervicales.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
+          <t>_REVISAR/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1846,19 +2518,19 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 14502216 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2FtAnGbLjjQrrdgRww'}</t>
+          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1rRgSwtQWA6h02p8yGoUlgmc6Qc3x6DsU/view</t>
+          <t>https://drive.google.com/file/d/1TCe5Bw2AmGt-EY4LEgt1cNaiWg-RwFLC/view</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>REVISAR_2020-07-14_nuclear_rastreo-yodo.pdf</t>
+          <t>REVISAR_2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -1867,12 +2539,12 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2020/radiologia/2020-07-14_nuclear_rastreo-yodo.pdf</t>
+          <t>2023/radiologia/2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-07-14_nuclear_rastreo-yodo.pdf</t>
+          <t>_REVISAR/REVISAR_2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1882,19 +2554,19 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 15897908 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2GRLmCKoVfim2sENBS'}</t>
+          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1rf96g6MjMv984xtt0QyWjjnklULtvj3N/view</t>
+          <t>https://drive.google.com/file/d/1FXbHPyQbqDHJOUMxnHiX_PjAFxFZ-3tH/view</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>REVISAR_2020-05-23_ultrasonido_cuello.pdf</t>
+          <t>REVISAR_2023-07-15_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -1903,12 +2575,12 @@
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2020/ultrasonidos/2020-05-23_ultrasonido_cuello.pdf</t>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-05-23_ultrasonido_cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2023-07-15_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1918,19 +2590,19 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 10838968 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2GndBhKpRcTJwPBgCs'}</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1z424DznUpGdbjwRU0dlzICuxFdSfVYW1/view</t>
+          <t>https://drive.google.com/file/d/1nVYop178pAvYlWWv2NAgn-gp4xxWnYEg/view</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
+          <t>REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -1939,12 +2611,12 @@
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2021/labs/2021-06-07_labs_quest-mx_biometria.pdf</t>
+          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
+          <t>_REVISAR/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1954,19 +2626,19 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 15699400 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2BhbBQmoVW98NVoAt8'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1CASli8xRI7Y1wLKR6oLBZ3JQRf-Y1KdU/view</t>
+          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
+          <t>REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -1975,12 +2647,12 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2021/labs/2021-06-07_labs_quest-mx_biometria_2.pdf</t>
+          <t>2024/radiologia/2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
+          <t>_REVISAR/REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1990,19 +2662,19 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 15699400 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2AgURyCKTqtuj8jxGa'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nuqeeVhX0deJ7BwXzsKAfsUsOPgi_HLF/view</t>
+          <t>https://drive.google.com/file/d/16xaHpUoMTXS17zDuCR9TG4nWF5YyvVkU/view</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>REVISAR_2021-12-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -2011,12 +2683,12 @@
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2021/labs/2021-12-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>2025/labs/2025-08-11_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2021-12-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2026,19 +2698,19 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 13852928 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2BB7rotVD6fLWYKLsa'}</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1biQ7aNiS2p3mTi15rbgT2OE1HBr6scUP/view</t>
+          <t>https://drive.google.com/file/d/1HMHksW_l3aF1lq9X3I0T0aSvDNNx3gpu/view</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>REVISAR_2021-12-22_ultrasonido_cuello.pdf</t>
+          <t>REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -2047,12 +2719,12 @@
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2021/ultrasonidos/2021-12-22_ultrasonido_cuello.pdf</t>
+          <t>2025/labs/2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2021-12-22_ultrasonido_cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2062,19 +2734,19 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 14199208 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2CDgvdMyWaZuAEiqGb'}</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1SB7Z_2GOg3VG7gV0fVUUXPj0gYamdbXo/view</t>
+          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -2083,12 +2755,12 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2022/labs/2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>2025/labs/2025-10-24_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>_REVISAR/REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2098,19 +2770,19 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 15547828 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW279YzkrNQSc6bxr6kP'}</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1UECfx-gSSTtlJVsvrEzkGi6uh5okeiN-/view</t>
+          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
+          <t>REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -2119,12 +2791,12 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
+          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2134,19 +2806,19 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 16602268 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW27kQyvAyZhYWvSQWJ2'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1yCWX0hgZnqKA57F22HZispDTzJKYOazt/view</t>
+          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>REVISAR_2022-06-06_ultrasonido_tiroides.pdf</t>
+          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -2155,12 +2827,12 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2022/ultrasonidos/2022-06-06_ultrasonido_tiroides.pdf</t>
+          <t>2026/labs/2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2022-06-06_ultrasonido_tiroides.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2170,19 +2842,19 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 16625592 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW28MxtmKczHxJbSkfRW'}</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1-rG8B2xpt-B6Okw5xi7AskcAYsnjOxiv/view</t>
+          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>REVISAR_2022-10-03_ultrasonido_cuello.pdf</t>
+          <t>REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -2191,12 +2863,12 @@
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
-          <t>2022/ultrasonidos/2022-10-03_ultrasonido_cuello.pdf</t>
+          <t>2026/radiologia/2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2022-10-03_ultrasonido_cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2206,516 +2878,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 14275604 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW28t9M4iAsY87MMC9mh'}</t>
+          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/11zttxbCEKhjP1KQWynf-lKor0LmoduHe/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr"/>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 15377456 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW1vmpG9HbWAsK9JE9ey'}</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1TCe5Bw2AmGt-EY4LEgt1cNaiWg-RwFLC/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>REVISAR_2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
-      <c r="D36" t="inlineStr"/>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>2023/radiologia/2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 19830012 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW1wPkVXUAxbb6DdK256'}</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1FXbHPyQbqDHJOUMxnHiX_PjAFxFZ-3tH/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>REVISAR_2023-07-15_ultrasonido_cuello.pdf</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonido_cuello.pdf</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2023-07-15_ultrasonido_cuello.pdf</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 19264496 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW1x45q974FwLb4sehT1'}</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1nVYop178pAvYlWWv2NAgn-gp4xxWnYEg/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 15103304 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2A5rpg56eSSZcu3MyS'}</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
-      <c r="D39" t="inlineStr"/>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>2024/radiologia/2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 15796452 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW29UN91TisaUDmUDj5R'}</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/16xaHpUoMTXS17zDuCR9TG4nWF5YyvVkU/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
-      <c r="D40" t="inlineStr"/>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>2025/labs/2025-08-11_labs_labcorp-ny_general.pdf</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 16503480 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2HQaQJ2AKJbqSbRmwY'}</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1HMHksW_l3aF1lq9X3I0T0aSvDNNx3gpu/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
-      <c r="D41" t="inlineStr"/>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>2025/labs/2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
-        </is>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 19316820 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2J69uaJka2wKaNSfjy'}</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
-      <c r="D42" t="inlineStr"/>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>2025/labs/2025-10-24_labs_labcorp-ny_general.pdf</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
-        </is>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 14749104 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2Jfxu6nKZwtGohZjQZ'}</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-05-25_inbody_mnc.jpg</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
-      <c r="D43" t="inlineStr"/>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>2026/inbody/2026-05-25_inbody_mnc.jpg</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-05-25_inbody_mnc.jpg</t>
-        </is>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Error code: 404 - {'type': 'error', 'error': {'type': 'not_found_error', 'message': 'model: claude-sonnet-4-20250514'}, 'request_id': 'req_011CeW2JnssXc51NCFyVwJYA'}</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1xsRRCzzETUWiVniCP37RdKGqnoAWf948/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>extraction failed (text): Error code: 404 - {'type': 'error', 'error': {'type': 'not_found_error', 'message': 'model: claude-sonnet-4-20250514'}, 'request_id': 'req_011CeW2Jyx8Q5FmGducgmDaL'}</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>2026/labs/2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 18366088 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2Knb2teuY3suQbwcuQ'}</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-04-17_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>2026/labs/2026-04-17_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-04-17_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>extraction failed (text): Error code: 404 - {'type': 'error', 'error': {'type': 'not_found_error', 'message': 'model: claude-sonnet-4-20250514'}, 'request_id': 'req_011CeW2K6diHwnrRJW29NQLe'}</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1UFeodi51jpRW9wcmxggZwTnSBr6yz8Yn/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
-      <c r="D47" t="inlineStr"/>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>2026/radiologia/2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 19367060 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2MApXzUPaZbjfiyQUE'}</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr">
-        <is>
           <t>https://drive.google.com/file/d/1XEJc1QCLZ_7qVoTuM_paOCfx8BblEA1e/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-04-14_ultrasonido_tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
-      <c r="D48" t="inlineStr"/>
-      <c r="E48" t="inlineStr"/>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonido_tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-04-14_ultrasonido_tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Error code: 400 - {'type': 'error', 'error': {'type': 'invalid_request_error', 'message': 'messages.0.content.0.image.source.base64: image exceeds 10 MB maximum: 19714500 bytes &gt; 10485760 bytes'}, 'request_id': 'req_011CeW2LUB2uJotta5kXhJC3'}</t>
-        </is>
-      </c>
-      <c r="J48" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1M2fSSCUpWpLLZ_bJAAfgT1LckEtoI9gE/view</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update master tracker 2026-08-29 00:12 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-28 23:54</t>
+          <t>2026-08-29 00:12</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -688,7 +688,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2019-03-18_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019-03-18_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -718,12 +718,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2019/labs/2019-03-18_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/labs/2019-03-18_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -1024,7 +1024,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1224,19 +1224,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1288,6 +1288,54 @@
       <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Drive Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2023-07-14_radiologia_hospital-angeles-pedregal_pet-ct.pdf</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2023-07-14</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>pet-ct</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2023/radiologia/2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2023/radiologia/2023-07-14_radiologia_hospital-angeles-pedregal_pet-ct.pdf</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1FXbHPyQbqDHJOUMxnHiX_PjAFxFZ-3tH/view</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1834,7 +1882,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -1906,7 +1954,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
+          <t>extraction failed (vision): no text content block in model response</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -2086,7 +2134,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>date: unparseable_date_text</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2122,7 +2170,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>extraction failed (vision): Unterminated string starting at: line 9 column 12 (char 228)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -2194,7 +2242,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
+          <t>extraction failed (vision): Unterminated string starting at: line 9 column 12 (char 223)</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -2338,7 +2386,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -2410,7 +2458,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -2518,7 +2566,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -2530,7 +2578,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>REVISAR_2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
+          <t>REVISAR_2023-07-15_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -2539,12 +2587,12 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2023/radiologia/2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
+          <t>_REVISAR/REVISAR_2023-07-15_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2554,19 +2602,19 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FXbHPyQbqDHJOUMxnHiX_PjAFxFZ-3tH/view</t>
+          <t>https://drive.google.com/file/d/1nVYop178pAvYlWWv2NAgn-gp4xxWnYEg/view</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>REVISAR_2023-07-15_ultrasonido_cuello.pdf</t>
+          <t>REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -2575,12 +2623,12 @@
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonido_cuello.pdf</t>
+          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2023-07-15_ultrasonido_cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2590,19 +2638,19 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>date: unparseable_date_text</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nVYop178pAvYlWWv2NAgn-gp4xxWnYEg/view</t>
+          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
+          <t>REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -2611,12 +2659,12 @@
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
+          <t>2024/radiologia/2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
+          <t>_REVISAR/REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2631,14 +2679,14 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
+          <t>https://drive.google.com/file/d/16xaHpUoMTXS17zDuCR9TG4nWF5YyvVkU/view</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
+          <t>REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -2647,12 +2695,12 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>2024/radiologia/2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2025/labs/2025-08-11_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
+          <t>_REVISAR/REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2662,19 +2710,19 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: unparseable_date_text</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/16xaHpUoMTXS17zDuCR9TG4nWF5YyvVkU/view</t>
+          <t>https://drive.google.com/file/d/1HMHksW_l3aF1lq9X3I0T0aSvDNNx3gpu/view</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
+          <t>REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -2683,12 +2731,12 @@
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
-          <t>2025/labs/2025-08-11_labs_labcorp-ny_general.pdf</t>
+          <t>2025/labs/2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
+          <t>_REVISAR/REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2703,14 +2751,14 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1HMHksW_l3aF1lq9X3I0T0aSvDNNx3gpu/view</t>
+          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
+          <t>REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -2719,12 +2767,12 @@
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
-          <t>2025/labs/2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
+          <t>2025/labs/2025-10-24_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
+          <t>_REVISAR/REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2739,14 +2787,14 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
+          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
+          <t>REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="B31" t="inlineStr"/>
@@ -2755,12 +2803,12 @@
       <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-24_labs_labcorp-ny_general.pdf</t>
+          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2770,19 +2818,19 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>date: unparseable_date_text</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
+          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -2791,12 +2839,12 @@
       <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
-          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
+          <t>2026/labs/2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2811,14 +2859,14 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
+          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
+          <t>REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="B33" t="inlineStr"/>
@@ -2827,12 +2875,12 @@
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
-          <t>2026/labs/2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
+          <t>2026/radiologia/2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2842,46 +2890,10 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>extraction failed (vision): no text content block in model response</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
-      <c r="D34" t="inlineStr"/>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>2026/radiologia/2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): 'ThinkingBlock' object has no attribute 'text'</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1XEJc1QCLZ_7qVoTuM_paOCfx8BblEA1e/view</t>
         </is>

</xml_diff>

<commit_message>
chore: update master tracker 2026-08-29 00:26 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29 00:12</t>
+          <t>2026-08-29 00:26</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>32</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -578,7 +578,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="56" customWidth="1" min="6" max="6"/>
     <col width="56" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
@@ -688,7 +688,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2019-03-18_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2019-03-18_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -718,12 +718,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2019/labs/2019-03-18_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2019/labs/2019-03-18_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -784,7 +784,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2019-05-15_labs_quest-mx_general-orina.pdf</t>
+          <t>2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>general-orina</t>
+          <t>general</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -832,7 +832,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019-09-13_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-lipidico</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -862,12 +862,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/labs/2019-09-13_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -1168,17 +1168,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-17_labs_quest-mx_general.pdf</t>
+          <t>2025-08-11_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2025-08-11</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>quest-mx</t>
+          <t>labcorp</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1188,17 +1188,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026/labs/2026-04-17_labs_quest-mx_biometria.pdf</t>
+          <t>2025/labs/2025-08-11_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026/labs/2026-04-17_labs_quest-mx_general.pdf</t>
+          <t>2025/labs/2025-08-11_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1208,6 +1208,150 @@
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1HMHksW_l3aF1lq9X3I0T0aSvDNNx3gpu/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>labcorp</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>tiroglobulina</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-10-23_labs_labcorp_general.pdf</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>labcorp</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-10-24_labs_labcorp-ny_general.pdf</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-17_labs_quest-mx_general.pdf</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026/labs/2026-04-17_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2026/labs/2026-04-17_labs_quest-mx_general.pdf</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1UFeodi51jpRW9wcmxggZwTnSBr6yz8Yn/view</t>
         </is>
@@ -1224,13 +1368,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -1294,37 +1438,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2023-07-14_radiologia_hospital-angeles-pedregal_pet-ct.pdf</t>
+          <t>2019-03-11_radiologia_hospital-san-angel-inn_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2023-07-14</t>
+          <t>2019-03-11</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>hospital-angeles-pedregal</t>
+          <t>hospital-san-angel-inn</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>pet-ct</t>
+          <t>rastreo-yodo</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2023/radiologia/2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2019/radiologia/2019-03-11_nuclear_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2023/radiologia/2023-07-14_radiologia_hospital-angeles-pedregal_pet-ct.pdf</t>
+          <t>2019/radiologia/2019-03-11_radiologia_hospital-san-angel-inn_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1334,6 +1478,102 @@
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1aia7BfJ-fw8149Vg-5iKgJZJ7g2IHK8l/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2020-07-14_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2020-07-14</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>rastreo-yodo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2020/radiologia/2020-07-14_nuclear_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2020/radiologia/2020-07-14_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1rf96g6MjMv984xtt0QyWjjnklULtvj3N/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2023-07-14_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2023-07-14</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2023/radiologia/2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2023/radiologia/2023-07-14_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1FXbHPyQbqDHJOUMxnHiX_PjAFxFZ-3tH/view</t>
         </is>
@@ -1350,12 +1590,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
@@ -1420,37 +1660,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2019-08-21_ultrasonidos_quest-mx_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2019-08-21</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>hospital-angeles-lomas</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ultrasonido-tiroides</t>
+          <t>ultrasonido-cuello</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonido_tiroides.pdf</t>
+          <t>2019/ultrasonidos/2019-08-21_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2019/ultrasonidos/2019-08-21_ultrasonidos_quest-mx_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1461,7 +1701,199 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1M2fSSCUpWpLLZ_bJAAfgT1LckEtoI9gE/view</t>
+          <t>https://drive.google.com/file/d/10vh3Q4UHpBkOWSKLZAkMTumYwzVgfypN/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2020-05-23_ultrasonidos_otro_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2020-05-23</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>otro</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>ultrasonido-tiroides</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2020/ultrasonidos/2020-05-23_ultrasonido_cuello.pdf</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2020/ultrasonidos/2020-05-23_ultrasonidos_otro_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1z424DznUpGdbjwRU0dlzICuxFdSfVYW1/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2021-12-22_ultrasonidos_quest-mx_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2021-12-22</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>ultrasonido-tiroides</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2021/ultrasonidos/2021-12-22_ultrasonido_cuello.pdf</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2021/ultrasonidos/2021-12-22_ultrasonidos_quest-mx_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1SB7Z_2GOg3VG7gV0fVUUXPj0gYamdbXo/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2022-06-06_ultrasonidos_quest-mx_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2022-06-06</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ultrasonido-tiroides</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2022/ultrasonidos/2022-06-06_ultrasonido_tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2022/ultrasonidos/2022-06-06_ultrasonidos_quest-mx_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1-rG8B2xpt-B6Okw5xi7AskcAYsnjOxiv/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2023-07-15</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>clinica-anahuac</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>ultrasonido-cuello</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonido_cuello.pdf</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1nVYop178pAvYlWWv2NAgn-gp4xxWnYEg/view</t>
         </is>
       </c>
     </row>
@@ -1479,10 +1911,10 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="53" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="39" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -1546,7 +1978,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-25_inbody_hospital-angeles-lomas_composicion-corporal.jpg</t>
+          <t>2026-05-25_inbody_hospital-angeles-lomas_inbody.jpg</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1561,7 +1993,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>composicion-corporal</t>
+          <t>inbody</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1576,7 +2008,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026/inbody/2026-05-25_inbody_hospital-angeles-lomas_composicion-corporal.jpg</t>
+          <t>2026/inbody/2026-05-25_inbody_hospital-angeles-lomas_inbody.jpg</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1602,19 +2034,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1666,6 +2098,102 @@
       <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Drive Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2018-12-24_patologia_hospital-satelite-dominguez-malagon_biopsia-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2018-12-24</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>hospital-satelite-dominguez-malagon</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>biopsia-tiroides</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2018/patologia/2018-12-24_patologia_metastasis-papilar.pdf</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2018/patologia/2018-12-24_patologia_hospital-satelite-dominguez-malagon_biopsia-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/17YnpChBP-Wq4Q3nCB9g5lk7n1STZAUcK/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2019-04-29</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mutacion-braf</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2019/radiologia/2019-04-29_patologia_braf-v600e.pdf</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1J4gLdlbUkRGF_aKpx6xqt-qvIimskL5x/view</t>
         </is>
       </c>
     </row>
@@ -1680,7 +2208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J33"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1750,7 +2278,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>REVISAR_2018-12-24_patologia_metastasis-papilar.pdf</t>
+          <t>REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -1759,12 +2287,12 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_metastasis-papilar.pdf</t>
+          <t>2019/labs/2019-04-12_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2018-12-24_patologia_metastasis-papilar.pdf</t>
+          <t>_REVISAR/REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1774,19 +2302,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date: unparseable_date_text</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17YnpChBP-Wq4Q3nCB9g5lk7n1STZAUcK/view</t>
+          <t>https://drive.google.com/file/d/10k9PIQTuP00FjD3--JFilIztJsAHzLex/view</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
+          <t>REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -1795,12 +2323,12 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2019/labs/2019-04-12_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/labs/2019-06-02_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1815,14 +2343,14 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/10k9PIQTuP00FjD3--JFilIztJsAHzLex/view</t>
+          <t>https://drive.google.com/file/d/1ffwqecdhzalYlS6o1XRwtznJRSrJ-KGV/view</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
+          <t>REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -1831,12 +2359,12 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2019/labs/2019-06-02_labs_quest-mx_general.pdf</t>
+          <t>2019/radiologia/2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
+          <t>_REVISAR/REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1851,14 +2379,14 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ffwqecdhzalYlS6o1XRwtznJRSrJ-KGV/view</t>
+          <t>https://drive.google.com/file/d/17PCU-FXw71gWbY5q8Id6_YjqM-d_BoVz/view</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
+          <t>REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -1867,12 +2395,12 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2019/radiologia/2019-01-09_patologia_diseccion-cuello.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
+          <t>_REVISAR/REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1887,14 +2415,14 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17PCU-FXw71gWbY5q8Id6_YjqM-d_BoVz/view</t>
+          <t>https://drive.google.com/file/d/1LYjog3waD7Oso0nAvtdOUpNEqfwYTmgY/view</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
+          <t>REVISAR_2019-08-21_rx_torax.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -1903,12 +2431,12 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-01-09_patologia_diseccion-cuello.pdf</t>
+          <t>2019/radiologia/2019-08-21_rx_torax.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2019-08-21_rx_torax.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1918,19 +2446,19 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>date: unparseable_date_text</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1LYjog3waD7Oso0nAvtdOUpNEqfwYTmgY/view</t>
+          <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>REVISAR_2019-03-11_nuclear_rastreo-yodo.pdf</t>
+          <t>REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -1939,12 +2467,12 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-03-11_nuclear_rastreo-yodo.pdf</t>
+          <t>2020/labs/2020-12-10_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-03-11_nuclear_rastreo-yodo.pdf</t>
+          <t>_REVISAR/REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1954,19 +2482,19 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>extraction failed (vision): no text content block in model response</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1aia7BfJ-fw8149Vg-5iKgJZJ7g2IHK8l/view</t>
+          <t>https://drive.google.com/file/d/1kkEH36xcggv0M0nYPQP1z7GX8a6d1Q-3/view</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>REVISAR_2019-04-29_patologia_braf-v600e.pdf</t>
+          <t>REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -1975,12 +2503,12 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-04-29_patologia_braf-v600e.pdf</t>
+          <t>2020/radiologia/2020-06-01_patologia_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-04-29_patologia_braf-v600e.pdf</t>
+          <t>_REVISAR/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1990,19 +2518,19 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>date: unparseable_date_text</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1J4gLdlbUkRGF_aKpx6xqt-qvIimskL5x/view</t>
+          <t>https://drive.google.com/file/d/19PXsFTn8Hf3QyTUKLZGk5MDFmI978hn4/view</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>REVISAR_2019-08-21_rx_torax.pdf</t>
+          <t>REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -2011,12 +2539,12 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-08-21_rx_torax.pdf</t>
+          <t>2020/radiologia/2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-08-21_rx_torax.pdf</t>
+          <t>_REVISAR/REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -2026,19 +2554,19 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>date: unparseable_date_text</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
+          <t>https://drive.google.com/file/d/1GcHOu5s7I3sn3A91BaqbSp0DkbtRu3tU/view</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>REVISAR_2019-08-21_ultrasonido_cuello.pdf</t>
+          <t>REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -2047,12 +2575,12 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2019/ultrasonidos/2019-08-21_ultrasonido_cuello.pdf</t>
+          <t>2020/radiologia/2020-06-05_patologia_ganglios-cervicales.pdf</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-08-21_ultrasonido_cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -2062,19 +2590,19 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>date: unparseable_date_text</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/10vh3Q4UHpBkOWSKLZAkMTumYwzVgfypN/view</t>
+          <t>https://drive.google.com/file/d/1rRgSwtQWA6h02p8yGoUlgmc6Qc3x6DsU/view</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
+          <t>REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -2083,12 +2611,12 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2020/labs/2020-12-10_labs_quest-mx_tiroideo.pdf</t>
+          <t>2021/labs/2021-06-07_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -2103,14 +2631,14 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1kkEH36xcggv0M0nYPQP1z7GX8a6d1Q-3/view</t>
+          <t>https://drive.google.com/file/d/1CASli8xRI7Y1wLKR6oLBZ3JQRf-Y1KdU/view</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
+          <t>REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -2119,12 +2647,12 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2020/radiologia/2020-06-01_patologia_baaf-ganglio.pdf</t>
+          <t>2021/labs/2021-06-07_labs_quest-mx_biometria_2.pdf</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
+          <t>_REVISAR/REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -2134,19 +2662,19 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>date: no_date_found</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/19PXsFTn8Hf3QyTUKLZGk5MDFmI978hn4/view</t>
+          <t>https://drive.google.com/file/d/1nuqeeVhX0deJ7BwXzsKAfsUsOPgi_HLF/view</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
+          <t>REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -2155,12 +2683,12 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2020/radiologia/2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2022/labs/2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
+          <t>_REVISAR/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2170,19 +2698,19 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Unterminated string starting at: line 9 column 12 (char 228)</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1GcHOu5s7I3sn3A91BaqbSp0DkbtRu3tU/view</t>
+          <t>https://drive.google.com/file/d/1UECfx-gSSTtlJVsvrEzkGi6uh5okeiN-/view</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
+          <t>REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr"/>
@@ -2191,12 +2719,12 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2020/radiologia/2020-06-05_patologia_ganglios-cervicales.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
+          <t>_REVISAR/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2206,19 +2734,19 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1rRgSwtQWA6h02p8yGoUlgmc6Qc3x6DsU/view</t>
+          <t>https://drive.google.com/file/d/1yCWX0hgZnqKA57F22HZispDTzJKYOazt/view</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>REVISAR_2020-07-14_nuclear_rastreo-yodo.pdf</t>
+          <t>REVISAR_2022-10-03_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -2227,12 +2755,12 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2020/radiologia/2020-07-14_nuclear_rastreo-yodo.pdf</t>
+          <t>2022/ultrasonidos/2022-10-03_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-07-14_nuclear_rastreo-yodo.pdf</t>
+          <t>_REVISAR/REVISAR_2022-10-03_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2242,19 +2770,19 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>extraction failed (vision): Unterminated string starting at: line 9 column 12 (char 223)</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1rf96g6MjMv984xtt0QyWjjnklULtvj3N/view</t>
+          <t>https://drive.google.com/file/d/11zttxbCEKhjP1KQWynf-lKor0LmoduHe/view</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>REVISAR_2020-05-23_ultrasonido_cuello.pdf</t>
+          <t>REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -2263,12 +2791,12 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2020/ultrasonidos/2020-05-23_ultrasonido_cuello.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-05-23_ultrasonido_cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2278,19 +2806,19 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>date: unparseable_date_text</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1z424DznUpGdbjwRU0dlzICuxFdSfVYW1/view</t>
+          <t>https://drive.google.com/file/d/1TCe5Bw2AmGt-EY4LEgt1cNaiWg-RwFLC/view</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
+          <t>REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -2299,12 +2827,12 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2021/labs/2021-06-07_labs_quest-mx_biometria.pdf</t>
+          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
+          <t>_REVISAR/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2319,14 +2847,14 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1CASli8xRI7Y1wLKR6oLBZ3JQRf-Y1KdU/view</t>
+          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
+          <t>REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -2335,12 +2863,12 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2021/labs/2021-06-07_labs_quest-mx_biometria_2.pdf</t>
+          <t>2024/radiologia/2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
+          <t>_REVISAR/REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2355,14 +2883,14 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nuqeeVhX0deJ7BwXzsKAfsUsOPgi_HLF/view</t>
+          <t>https://drive.google.com/file/d/16xaHpUoMTXS17zDuCR9TG4nWF5YyvVkU/view</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>REVISAR_2021-12-22_ultrasonido_cuello.pdf</t>
+          <t>REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -2371,12 +2899,12 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2021/ultrasonidos/2021-12-22_ultrasonido_cuello.pdf</t>
+          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2021-12-22_ultrasonido_cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2386,19 +2914,19 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>date: unparseable_date_text</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1SB7Z_2GOg3VG7gV0fVUUXPj0gYamdbXo/view</t>
+          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -2407,12 +2935,12 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2022/labs/2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>2026/labs/2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2427,14 +2955,14 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1UECfx-gSSTtlJVsvrEzkGi6uh5okeiN-/view</t>
+          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
+          <t>REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -2443,12 +2971,12 @@
       <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
+          <t>2026/radiologia/2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2458,19 +2986,19 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>date: no_date_found</t>
+          <t>date: ambiguous_day_month</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1yCWX0hgZnqKA57F22HZispDTzJKYOazt/view</t>
+          <t>https://drive.google.com/file/d/1XEJc1QCLZ_7qVoTuM_paOCfx8BblEA1e/view</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>REVISAR_2022-06-06_ultrasonido_tiroides.pdf</t>
+          <t>REVISAR_2026-04-14_ultrasonido_tiroides.pdf</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -2479,12 +3007,12 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2022/ultrasonidos/2022-06-06_ultrasonido_tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonido_tiroides.pdf</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2022-06-06_ultrasonido_tiroides.pdf</t>
+          <t>_REVISAR/REVISAR_2026-04-14_ultrasonido_tiroides.pdf</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2494,408 +3022,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>date: unparseable_date_text</t>
+          <t>extraction failed (vision): Unterminated string starting at: line 9 column 12 (char 244)</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1-rG8B2xpt-B6Okw5xi7AskcAYsnjOxiv/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>REVISAR_2022-10-03_ultrasonido_cuello.pdf</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>2022/ultrasonidos/2022-10-03_ultrasonido_cuello.pdf</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2022-10-03_ultrasonido_cuello.pdf</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/11zttxbCEKhjP1KQWynf-lKor0LmoduHe/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>date: no_date_found</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1TCe5Bw2AmGt-EY4LEgt1cNaiWg-RwFLC/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>REVISAR_2023-07-15_ultrasonido_cuello.pdf</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonido_cuello.pdf</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2023-07-15_ultrasonido_cuello.pdf</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>date: unparseable_date_text</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1nVYop178pAvYlWWv2NAgn-gp4xxWnYEg/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>2024/radiologia/2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/16xaHpUoMTXS17zDuCR9TG4nWF5YyvVkU/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>2025/labs/2025-08-11_labs_labcorp-ny_general.pdf</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>date: unparseable_date_text</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1HMHksW_l3aF1lq9X3I0T0aSvDNNx3gpu/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>2025/labs/2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>date: unparseable_date_text</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>2025/labs/2025-10-24_labs_labcorp-ny_general.pdf</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>date: unparseable_date_text</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>2026/labs/2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I32" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>2026/radiologia/2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): no text content block in model response</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1XEJc1QCLZ_7qVoTuM_paOCfx8BblEA1e/view</t>
+          <t>https://drive.google.com/file/d/1M2fSSCUpWpLLZ_bJAAfgT1LckEtoI9gE/view</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update master tracker 2026-08-29 00:38 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29 00:26</t>
+          <t>2026-08-29 00:38</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -832,7 +832,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2019-09-13_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019-09-13_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -847,7 +847,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>perfil-lipidico</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -862,12 +862,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2019/labs/2019-09-13_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -1024,7 +1024,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1590,12 +1590,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
@@ -1852,7 +1852,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
+          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ultrasonido-cuello</t>
+          <t>ultrasonido-tiroides</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1894,6 +1894,54 @@
       <c r="J6" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1nVYop178pAvYlWWv2NAgn-gp4xxWnYEg/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>hospital-angeles-lomas</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>ultrasonido-tiroides</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonido_tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1M2fSSCUpWpLLZ_bJAAfgT1LckEtoI9gE/view</t>
         </is>
       </c>
     </row>
@@ -1911,10 +1959,10 @@
   <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="53" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="39" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -1978,7 +2026,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-25_inbody_hospital-angeles-lomas_inbody.jpg</t>
+          <t>2026-05-25_inbody_hospital-angeles-lomas_composicion-corporal.jpg</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1993,7 +2041,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>inbody</t>
+          <t>composicion-corporal</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -2008,7 +2056,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026/inbody/2026-05-25_inbody_hospital-angeles-lomas_inbody.jpg</t>
+          <t>2026/inbody/2026-05-25_inbody_hospital-angeles-lomas_composicion-corporal.jpg</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2208,7 +2256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2219,7 +2267,7 @@
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -2995,42 +3043,6 @@
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-04-14_ultrasonido_tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonido_tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-04-14_ultrasonido_tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>extraction failed (vision): Unterminated string starting at: line 9 column 12 (char 244)</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1M2fSSCUpWpLLZ_bJAAfgT1LckEtoI9gE/view</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: update master tracker 2026-08-29 00:58 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29 00:38</t>
+          <t>2026-08-29 00:58</t>
         </is>
       </c>
     </row>
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -526,7 +526,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1024,7 +1024,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1039,7 +1039,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1264,7 +1264,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1279,7 +1279,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1368,7 +1368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1379,7 +1379,7 @@
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -1438,22 +1438,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2019-03-11_radiologia_hospital-san-angel-inn_rastreo-yodo.pdf</t>
+          <t>2019-08-21_radiologia_quest-mx_torax.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2019-03-11</t>
+          <t>2019-08-21</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>hospital-san-angel-inn</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>rastreo-yodo</t>
+          <t>torax</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1463,12 +1463,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-03-11_nuclear_rastreo-yodo.pdf</t>
+          <t>2019/radiologia/2019-08-21_rx_torax.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-03-11_radiologia_hospital-san-angel-inn_rastreo-yodo.pdf</t>
+          <t>2019/radiologia/2019-08-21_radiologia_quest-mx_torax.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1479,7 +1479,7 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1aia7BfJ-fw8149Vg-5iKgJZJ7g2IHK8l/view</t>
+          <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
         </is>
       </c>
     </row>
@@ -1576,6 +1576,58 @@
       <c r="J4" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1FXbHPyQbqDHJOUMxnHiX_PjAFxFZ-3tH/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2024-08-12_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2024-08-12</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2024/radiologia/2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2024/radiologia/2024-08-12_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>date order inferred from 2nd date on same document ('13/08/2024', unambiguous as DM) — '12/08/2024' itself was ambiguous</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/16xaHpUoMTXS17zDuCR9TG4nWF5YyvVkU/view</t>
         </is>
       </c>
     </row>
@@ -1590,18 +1642,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -1804,17 +1856,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2022-06-06_ultrasonidos_quest-mx_ultrasonido-tiroides.pdf</t>
+          <t>2022-03-10_ultrasonidos_envision-imaging_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2022-06-06</t>
+          <t>2022-03-10</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>quest-mx</t>
+          <t>envision-imaging</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1829,12 +1881,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2022/ultrasonidos/2022-06-06_ultrasonido_tiroides.pdf</t>
+          <t>2022/ultrasonidos/2022-10-03_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2022/ultrasonidos/2022-06-06_ultrasonidos_quest-mx_ultrasonido-tiroides.pdf</t>
+          <t>2022/ultrasonidos/2022-03-10_ultrasonidos_envision-imaging_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1842,27 +1894,31 @@
           <t>rename</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>date order inferred from 2nd date on same document ('5/20/2020', unambiguous as MD) — '3/10/2022' itself was ambiguous</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1-rG8B2xpt-B6Okw5xi7AskcAYsnjOxiv/view</t>
+          <t>https://drive.google.com/file/d/11zttxbCEKhjP1KQWynf-lKor0LmoduHe/view</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
+          <t>2022-06-06_ultrasonidos_quest-mx_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2023-07-15</t>
+          <t>2022-06-06</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>clinica-anahuac</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1872,17 +1928,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonido_cuello.pdf</t>
+          <t>2022/ultrasonidos/2022-06-06_ultrasonido_tiroides.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
+          <t>2022/ultrasonidos/2022-06-06_ultrasonidos_quest-mx_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1893,44 +1949,44 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nVYop178pAvYlWWv2NAgn-gp4xxWnYEg/view</t>
+          <t>https://drive.google.com/file/d/1-rG8B2xpt-B6Okw5xi7AskcAYsnjOxiv/view</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2023-07-15</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>hospital-angeles-lomas</t>
+          <t>clinica-anahuac</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ultrasonido-tiroides</t>
+          <t>ultrasonido-cuello</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonido_tiroides.pdf</t>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonido_cuello.pdf</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1940,6 +1996,54 @@
       </c>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1nVYop178pAvYlWWv2NAgn-gp4xxWnYEg/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ultrasonido-tiroides</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonido_tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1M2fSSCUpWpLLZ_bJAAfgT1LckEtoI9gE/view</t>
         </is>
@@ -2087,8 +2191,8 @@
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="37" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -2152,7 +2256,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_hospital-satelite-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dr-dominguez-malagon_inmunohistoquimica-tiroides.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2162,12 +2266,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>hospital-satelite-dominguez-malagon</t>
+          <t>dr-dominguez-malagon</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>biopsia-tiroides</t>
+          <t>inmunohistoquimica-tiroides</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -2182,7 +2286,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_hospital-satelite-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_inmunohistoquimica-tiroides.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2200,7 +2304,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
+          <t>2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2215,7 +2319,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>mutacion-braf</t>
+          <t>biopsia-tiroides</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -2230,7 +2334,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
+          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -2256,7 +2360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2267,7 +2371,7 @@
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="27" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -2350,7 +2454,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('4/12/2019') this is either 2019-12-04 (day-first) or 2019-04-12 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2386,7 +2490,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('2/06/2019') this is either 2019-06-02 (day-first) or 2019-02-06 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -2422,7 +2526,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('07/01/2019') this is either 2019-01-07 (day-first) or 2019-07-01 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -2458,7 +2562,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('09-01-19') this is either 2019-01-09 (day-first) or 2019-09-01 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -2470,7 +2574,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>REVISAR_2019-08-21_rx_torax.pdf</t>
+          <t>REVISAR_2019-03-11_nuclear_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -2479,12 +2583,12 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-08-21_rx_torax.pdf</t>
+          <t>2019/radiologia/2019-03-11_nuclear_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-08-21_rx_torax.pdf</t>
+          <t>_REVISAR/REVISAR_2019-03-11_nuclear_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2499,7 +2603,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
+          <t>https://drive.google.com/file/d/1aia7BfJ-fw8149Vg-5iKgJZJ7g2IHK8l/view</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2634,7 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('10/12/2020') this is either 2020-12-10 (day-first) or 2020-10-12 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -2602,7 +2706,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('02/06/2020') this is either 2020-06-02 (day-first) or 2020-02-06 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -2638,7 +2742,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('05-06-2020') this is either 2020-06-05 (day-first) or 2020-05-06 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -2674,7 +2778,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('07/06/2021') this is either 2021-06-07 (day-first) or 2021-07-06 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2710,7 +2814,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('07/06/2021') this is either 2021-06-07 (day-first) or 2021-07-06 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2746,7 +2850,7 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('03/09/2022') this is either 2022-09-03 (day-first) or 2022-03-09 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -2794,7 +2898,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>REVISAR_2022-10-03_ultrasonido_cuello.pdf</t>
+          <t>REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -2803,12 +2907,12 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2022/ultrasonidos/2022-10-03_ultrasonido_cuello.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2022-10-03_ultrasonido_cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2818,19 +2922,19 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/11zttxbCEKhjP1KQWynf-lKor0LmoduHe/view</t>
+          <t>https://drive.google.com/file/d/1TCe5Bw2AmGt-EY4LEgt1cNaiWg-RwFLC/view</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -2839,12 +2943,12 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>_REVISAR/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2854,19 +2958,19 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>date: no_date_found</t>
+          <t>date: ambiguous_day_month — as printed ('10/08/2024 9:38 AM') this is either 2024-08-10 (day-first) or 2024-10-08 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1TCe5Bw2AmGt-EY4LEgt1cNaiWg-RwFLC/view</t>
+          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
+          <t>REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -2875,12 +2979,12 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
+          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2890,19 +2994,19 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('05/03/2026') this is either 2026-03-05 (day-first) or 2026-05-03 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
+          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
+          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -2911,12 +3015,12 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2024/radiologia/2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2026/labs/2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2926,19 +3030,19 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('05/03/2026') this is either 2026-03-05 (day-first) or 2026-05-03 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/16xaHpUoMTXS17zDuCR9TG4nWF5YyvVkU/view</t>
+          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
+          <t>REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -2947,12 +3051,12 @@
       <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
+          <t>2026/radiologia/2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2962,82 +3066,10 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month</t>
+          <t>date: ambiguous_day_month — as printed ('06/03/2026') this is either 2026-03-06 (day-first) or 2026-06-03 (month-first); open the file to see which</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>2026/labs/2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>2026/radiologia/2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1XEJc1QCLZ_7qVoTuM_paOCfx8BblEA1e/view</t>
         </is>

</xml_diff>

<commit_message>
chore: update master tracker 2026-08-29 02:53 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29 00:58</t>
+          <t>2026-08-29 02:53</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>18</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -570,18 +570,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="56" customWidth="1" min="6" max="6"/>
-    <col width="56" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -784,12 +784,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019-04-12_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2019-05-15</t>
+          <t>2019-04-12</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -809,35 +809,39 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_orina.pdf</t>
+          <t>2019/labs/2019-04-12_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019/labs/2019-04-12_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr"/>
+          <t>no_change</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('2019-04-12_labs_quest-mx_tiroideo.pdf') — '4/12/2019' was ambiguous on its own, but the current name already matches the month-first reading</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1HIIPFPUwJQdLc9Qi-rUbP-wOLn8SRXtA/view</t>
+          <t>https://drive.google.com/file/d/10k9PIQTuP00FjD3--JFilIztJsAHzLex/view</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2019-09-13</t>
+          <t>2019-05-15</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -847,7 +851,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>general</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -857,35 +861,35 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_orina.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1txD2M8pAnAInDxjvL3pi712wRwmPTsPT/view</t>
+          <t>https://drive.google.com/file/d/1HIIPFPUwJQdLc9Qi-rUbP-wOLn8SRXtA/view</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2019-12-24_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019-06-02_labs_quest-mx_calcio.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2019-12-24</t>
+          <t>2019-06-02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -895,7 +899,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>perfil-lipidico</t>
+          <t>calcio</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -905,12 +909,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2019/labs/2019-12-24_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/labs/2019-06-02_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2019/labs/2019-12-24_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019/labs/2019-06-02_labs_quest-mx_calcio.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -918,22 +922,26 @@
           <t>rename</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('2019-06-02_labs_quest-mx_general.pdf') — '2/06/2019' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1qiH2_frLbKJ2vF2j6ICW6j9SRmbxxGU0/view</t>
+          <t>https://drive.google.com/file/d/1ffwqecdhzalYlS6o1XRwtznJRSrJ-KGV/view</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2020-04-17_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019-09-13_labs_quest-mx_perfil-tiroideo-lipidico.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2020-04-17</t>
+          <t>2019-09-13</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -943,22 +951,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>perfil-lipidico</t>
+          <t>perfil-tiroideo-lipidico</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2020/labs/2020-04-17_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2020/labs/2020-04-17_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019/labs/2019-09-13_labs_quest-mx_perfil-tiroideo-lipidico.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -969,19 +977,19 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1pdBluP-dzl_wE0f_FWKaNH-l1mFrxZvw/view</t>
+          <t>https://drive.google.com/file/d/1txD2M8pAnAInDxjvL3pi712wRwmPTsPT/view</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2020-04-28_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019-12-24_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2020-04-28</t>
+          <t>2019-12-24</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -996,17 +1004,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2020/labs/2020-04-28_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/labs/2019-12-24_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2020/labs/2020-04-28_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019/labs/2019-12-24_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1017,19 +1025,19 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1JIAoEhyttwxc6Cv_SHEYfi9jodXjI9R7/view</t>
+          <t>https://drive.google.com/file/d/1qiH2_frLbKJ2vF2j6ICW6j9SRmbxxGU0/view</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020-04-17_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2020-05-25</t>
+          <t>2020-04-17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1039,7 +1047,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-lipidico</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1049,12 +1057,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>2020/labs/2020-04-17_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/labs/2020-04-17_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1065,19 +1073,19 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1sNLAT_auII9ux0kE0dNzDNi-5cmWi4H_/view</t>
+          <t>https://drive.google.com/file/d/1pdBluP-dzl_wE0f_FWKaNH-l1mFrxZvw/view</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2020-06-15_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020-04-28_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2020-06-15</t>
+          <t>2020-04-28</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1087,7 +1095,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-lipidico</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1097,12 +1105,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2020/labs/2020-06-15_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>2020/labs/2020-04-28_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2020/labs/2020-06-15_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/labs/2020-04-28_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1113,19 +1121,19 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1xq4z67ZNSeS-Ir5m3rtl17ElitnuZ2j4/view</t>
+          <t>https://drive.google.com/file/d/1JIAoEhyttwxc6Cv_SHEYfi9jodXjI9R7/view</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2021-12-22_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2021-12-22</t>
+          <t>2020-05-25</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1135,22 +1143,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>perfil-lipidico</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2021/labs/2021-12-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2021/labs/2021-12-22_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1161,44 +1169,44 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1biQ7aNiS2p3mTi15rbgT2OE1HBr6scUP/view</t>
+          <t>https://drive.google.com/file/d/1sNLAT_auII9ux0kE0dNzDNi-5cmWi4H_/view</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025-08-11_labs_labcorp_general.pdf</t>
+          <t>2020-06-15_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2025-08-11</t>
+          <t>2020-06-15</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>labcorp</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2025/labs/2025-08-11_labs_labcorp-ny_general.pdf</t>
+          <t>2020/labs/2020-06-15_labs_quest-mx_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2025/labs/2025-08-11_labs_labcorp_general.pdf</t>
+          <t>2020/labs/2020-06-15_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1209,44 +1217,44 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1HMHksW_l3aF1lq9X3I0T0aSvDNNx3gpu/view</t>
+          <t>https://drive.google.com/file/d/1xq4z67ZNSeS-Ir5m3rtl17ElitnuZ2j4/view</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2020-12-10_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2020-12-10</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>labcorp</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>tiroglobulina</t>
+          <t>perfil-lipidico</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2025/labs/2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
+          <t>2020/labs/2020-12-10_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2020/labs/2020-12-10_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1254,70 +1262,78 @@
           <t>rename</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_tiroideo.pdf') — '10/12/2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
+          <t>https://drive.google.com/file/d/1kkEH36xcggv0M0nYPQP1z7GX8a6d1Q-3/view</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2021-06-07_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2021-06-07</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>labcorp</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>biometria</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-24_labs_labcorp-ny_general.pdf</t>
+          <t>2021/labs/2021-06-07_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2021/labs/2021-06-07_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>rename</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr"/>
+          <t>no_change</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('2021-06-07_labs_quest-mx_biometria.pdf') — '07/06/2021' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+          <t>https://drive.google.com/file/d/1CASli8xRI7Y1wLKR6oLBZ3JQRf-Y1KdU/view</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-17_labs_quest-mx_general.pdf</t>
+          <t>2021-12-22_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2021-12-22</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1327,22 +1343,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>perfil-lipidico</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026/labs/2026-04-17_labs_quest-mx_biometria.pdf</t>
+          <t>2021/labs/2021-12-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026/labs/2026-04-17_labs_quest-mx_general.pdf</t>
+          <t>2021/labs/2021-12-22_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1352,6 +1368,302 @@
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1biQ7aNiS2p3mTi15rbgT2OE1HBr6scUP/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2024-08-10_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2024-08-10</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>biometria</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>no_change</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-08-11_labs_labcorp_general.pdf</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2025-08-11</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>labcorp</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-08-11_labs_labcorp-ny_general.pdf</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-08-11_labs_labcorp_general.pdf</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1HMHksW_l3aF1lq9X3I0T0aSvDNNx3gpu/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>labcorp</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>tiroglobulina</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-10-23_labs_labcorp_general.pdf</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>labcorp</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-10-24_labs_labcorp-ny_general.pdf</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-05_labs_hospital-angeles-lomas_general.pdf</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>hospital-angeles-lomas</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_general.pdf</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('2026-03-05_labs_hospital-angeles-lomas_biometria.pdf') — '05/03/2026' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-17_labs_quest-mx_general.pdf</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026/labs/2026-04-17_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026/labs/2026-04-17_labs_quest-mx_general.pdf</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1UFeodi51jpRW9wcmxggZwTnSBr6yz8Yn/view</t>
         </is>
@@ -1368,7 +1680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1438,22 +1750,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2019-08-21_radiologia_quest-mx_torax.pdf</t>
+          <t>2019-01-07_radiologia_hospital-angeles-pedregal_pet.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2019-08-21</t>
+          <t>2019-01-07</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>quest-mx</t>
+          <t>hospital-angeles-pedregal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>torax</t>
+          <t>pet</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1463,12 +1775,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-08-21_rx_torax.pdf</t>
+          <t>2019/radiologia/2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-08-21_radiologia_quest-mx_torax.pdf</t>
+          <t>2019/radiologia/2019-01-07_radiologia_hospital-angeles-pedregal_pet.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1476,27 +1788,31 @@
           <t>rename</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('2019-01-07_pet_hospital-angeles-pedregal.pdf') — '07/01/2019' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
+          <t>https://drive.google.com/file/d/17PCU-FXw71gWbY5q8Id6_YjqM-d_BoVz/view</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2020-07-14_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+          <t>2019-03-11_radiologia_hospital-san-angel-inn_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2020-07-14</t>
+          <t>2019-03-11</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>hospital-angeles-pedregal</t>
+          <t>hospital-san-angel-inn</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1506,17 +1822,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2020/radiologia/2020-07-14_nuclear_rastreo-yodo.pdf</t>
+          <t>2019/radiologia/2019-03-11_nuclear_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2020/radiologia/2020-07-14_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+          <t>2019/radiologia/2019-03-11_radiologia_hospital-san-angel-inn_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1527,44 +1843,44 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1rf96g6MjMv984xtt0QyWjjnklULtvj3N/view</t>
+          <t>https://drive.google.com/file/d/1aia7BfJ-fw8149Vg-5iKgJZJ7g2IHK8l/view</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2023-07-14_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+          <t>2019-08-21_radiologia_quest-mx_torax.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2023-07-14</t>
+          <t>2019-08-21</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>hospital-angeles-pedregal</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>pet</t>
+          <t>torax</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2023/radiologia/2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2019/radiologia/2019-08-21_rx_torax.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2023/radiologia/2023-07-14_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+          <t>2019/radiologia/2019-08-21_radiologia_quest-mx_torax.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1575,59 +1891,259 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FXbHPyQbqDHJOUMxnHiX_PjAFxFZ-3tH/view</t>
+          <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>2020-06-02_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2020-06-02</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2020/radiologia/2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2020/radiologia/2020-06-02_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('2020-06-02_pet_hospital-angeles-pedregal.pdf') — '02/06/2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1GcHOu5s7I3sn3A91BaqbSp0DkbtRu3tU/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2020-07-14_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2020-07-14</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>rastreo-yodo</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2020/radiologia/2020-07-14_nuclear_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2020/radiologia/2020-07-14_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1rf96g6MjMv984xtt0QyWjjnklULtvj3N/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2023-07-14_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2023-07-14</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2023/radiologia/2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2023/radiologia/2023-07-14_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1FXbHPyQbqDHJOUMxnHiX_PjAFxFZ-3tH/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>2024-08-12_radiologia_hospital-angeles-pedregal_pet.pdf</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>2024-08-12</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>hospital-angeles-pedregal</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>pet</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>2024/radiologia/2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>2024/radiologia/2024-08-12_radiologia_hospital-angeles-pedregal_pet.pdf</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>rename</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>date order inferred from 2nd date on same document ('13/08/2024', unambiguous as DM) — '12/08/2024' itself was ambiguous</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/16xaHpUoMTXS17zDuCR9TG4nWF5YyvVkU/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-06_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>rastreo-yodo</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026/radiologia/2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026/radiologia/2026-03-06_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('2026-03-06_pet_hospital-angeles-pedregal.pdf') — '06/03/2026' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1XEJc1QCLZ_7qVoTuM_paOCfx8BblEA1e/view</t>
         </is>
       </c>
     </row>
@@ -1647,7 +2163,7 @@
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
@@ -2004,7 +2520,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2014,7 +2530,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>hospital-angeles-pedregal</t>
+          <t>hospital-angeles</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2034,7 +2550,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2186,18 +2702,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -2256,7 +2772,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_dr-dominguez-malagon_inmunohistoquimica-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2271,7 +2787,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>inmunohistoquimica-tiroides</t>
+          <t>biopsia-tiroides</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -2286,7 +2802,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_inmunohistoquimica-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2304,48 +2820,152 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2019-01-09_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2019-01-09</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>biopsia-tiroides</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2019/radiologia/2019-01-09_patologia_diseccion-cuello.pdf</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2019/patologia/2019-01-09_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('2019-01-09_patologia_diseccion-cuello.pdf') — '09-01-19' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1LYjog3waD7Oso0nAvtdOUpNEqfwYTmgY/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>2019-04-29</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>hospital-angeles-pedregal</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>biopsia-tiroides</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>2019/radiologia/2019-04-29_patologia_braf-v600e.pdf</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>move</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1J4gLdlbUkRGF_aKpx6xqt-qvIimskL5x/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2020-06-05</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>biopsia-tiroides</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2020/radiologia/2020-06-05_patologia_ganglios-cervicales.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('2020-06-05_patologia_ganglios-cervicales.pdf') — '05-06-2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1rRgSwtQWA6h02p8yGoUlgmc6Qc3x6DsU/view</t>
         </is>
       </c>
     </row>
@@ -2360,13 +2980,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -2430,7 +3050,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
+          <t>REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -2439,12 +3059,12 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2019/labs/2019-04-12_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/radiologia/2020-06-01_patologia_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2454,19 +3074,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month — as printed ('4/12/2019') this is either 2019-12-04 (day-first) or 2019-04-12 (month-first); open the file to see which</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/10k9PIQTuP00FjD3--JFilIztJsAHzLex/view</t>
+          <t>https://drive.google.com/file/d/19PXsFTn8Hf3QyTUKLZGk5MDFmI978hn4/view</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
+          <t>REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -2475,12 +3095,12 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2019/labs/2019-06-02_labs_quest-mx_general.pdf</t>
+          <t>2022/labs/2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
+          <t>_REVISAR/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -2490,19 +3110,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month — as printed ('2/06/2019') this is either 2019-06-02 (day-first) or 2019-02-06 (month-first); open the file to see which</t>
+          <t>date: ambiguous_day_month — as printed ('03/09/2022') this is either 2022-09-03 (day-first) or 2022-03-09 (month-first); open the file to see which (note: current filename implies 2022-10-03, which matches NEITHER reading — worth a closer look)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ffwqecdhzalYlS6o1XRwtznJRSrJ-KGV/view</t>
+          <t>https://drive.google.com/file/d/1UECfx-gSSTtlJVsvrEzkGi6uh5okeiN-/view</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
+          <t>REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -2511,12 +3131,12 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
+          <t>_REVISAR/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -2526,19 +3146,19 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month — as printed ('07/01/2019') this is either 2019-01-07 (day-first) or 2019-07-01 (month-first); open the file to see which</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17PCU-FXw71gWbY5q8Id6_YjqM-d_BoVz/view</t>
+          <t>https://drive.google.com/file/d/1yCWX0hgZnqKA57F22HZispDTzJKYOazt/view</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
+          <t>REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -2547,12 +3167,12 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-01-09_patologia_diseccion-cuello.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -2562,19 +3182,19 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month — as printed ('09-01-19') this is either 2019-01-09 (day-first) or 2019-09-01 (month-first); open the file to see which</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1LYjog3waD7Oso0nAvtdOUpNEqfwYTmgY/view</t>
+          <t>https://drive.google.com/file/d/1TCe5Bw2AmGt-EY4LEgt1cNaiWg-RwFLC/view</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>REVISAR_2019-03-11_nuclear_rastreo-yodo.pdf</t>
+          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -2583,12 +3203,12 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-03-11_nuclear_rastreo-yodo.pdf</t>
+          <t>2026/labs/2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-03-11_nuclear_rastreo-yodo.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2598,480 +3218,64 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>date: no_date_found</t>
+          <t>date: ambiguous_day_month — as printed ('05/03/2026') this is either 2026-03-05 (day-first) or 2026-05-03 (month-first); open the file to see which (note: current filename implies 2026-03-06, which matches NEITHER reading — worth a closer look)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1aia7BfJ-fw8149Vg-5iKgJZJ7g2IHK8l/view</t>
+          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+          <t>DUP_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2021-06-07</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>biometria</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2020/labs/2020-12-10_labs_quest-mx_tiroideo.pdf</t>
+          <t>2021/labs/2021-06-07_labs_quest-mx_biometria_2.pdf</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/DUP_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>quarantine</t>
+          <t>duplicate</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month — as printed ('10/12/2020') this is either 2020-12-10 (day-first) or 2020-10-12 (month-first); open the file to see which</t>
+          <t>duplicate of 2021/labs/2021-06-07_labs_quest-mx_biometria.pdf (identical content hash)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1kkEH36xcggv0M0nYPQP1z7GX8a6d1Q-3/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2020/radiologia/2020-06-01_patologia_baaf-ganglio.pdf</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>date: no_date_found</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/19PXsFTn8Hf3QyTUKLZGk5MDFmI978hn4/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2020/radiologia/2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('02/06/2020') this is either 2020-06-02 (day-first) or 2020-02-06 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1GcHOu5s7I3sn3A91BaqbSp0DkbtRu3tU/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2020/radiologia/2020-06-05_patologia_ganglios-cervicales.pdf</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('05-06-2020') this is either 2020-06-05 (day-first) or 2020-05-06 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1rRgSwtQWA6h02p8yGoUlgmc6Qc3x6DsU/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>2021/labs/2021-06-07_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('07/06/2021') this is either 2021-06-07 (day-first) or 2021-07-06 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1CASli8xRI7Y1wLKR6oLBZ3JQRf-Y1KdU/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>2021/labs/2021-06-07_labs_quest-mx_biometria_2.pdf</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('07/06/2021') this is either 2021-06-07 (day-first) or 2021-07-06 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
           <t>https://drive.google.com/file/d/1nuqeeVhX0deJ7BwXzsKAfsUsOPgi_HLF/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>2022/labs/2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('03/09/2022') this is either 2022-09-03 (day-first) or 2022-03-09 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1UECfx-gSSTtlJVsvrEzkGi6uh5okeiN-/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>date: no_date_found</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1yCWX0hgZnqKA57F22HZispDTzJKYOazt/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>date: no_date_found</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1TCe5Bw2AmGt-EY4LEgt1cNaiWg-RwFLC/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('10/08/2024 9:38 AM') this is either 2024-08-10 (day-first) or 2024-10-08 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('05/03/2026') this is either 2026-03-05 (day-first) or 2026-05-03 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>2026/labs/2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('05/03/2026') this is either 2026-03-05 (day-first) or 2026-05-03 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>2026/radiologia/2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('06/03/2026') this is either 2026-03-06 (day-first) or 2026-06-03 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1XEJc1QCLZ_7qVoTuM_paOCfx8BblEA1e/view</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update master tracker 2026-08-29 15:47 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29 15:34</t>
+          <t>2026-08-29 15:47</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -516,7 +516,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>19</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -570,18 +570,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="56" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -784,12 +784,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019-04-12_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2019-05-15</t>
+          <t>2019-04-12</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -799,7 +799,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -809,12 +809,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2019-05-15_labs_quest-mx_orina.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019/labs/2019-04-12_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -822,22 +822,26 @@
           <t>move</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf') — '4/12/2019' was ambiguous on its own, but the current name already matches the month-first reading</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1HIIPFPUwJQdLc9Qi-rUbP-wOLn8SRXtA/view</t>
+          <t>https://drive.google.com/file/d/10k9PIQTuP00FjD3--JFilIztJsAHzLex/view</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2019-09-13</t>
+          <t>2019-05-15</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -847,7 +851,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>general</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -857,12 +861,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2019-05-15_labs_quest-mx_orina.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -873,19 +877,19 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1txD2M8pAnAInDxjvL3pi712wRwmPTsPT/view</t>
+          <t>https://drive.google.com/file/d/1HIIPFPUwJQdLc9Qi-rUbP-wOLn8SRXtA/view</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2019-12-24_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019-06-02_labs_quest-mx_calcio.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2019-12-24</t>
+          <t>2019-06-02</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -895,7 +899,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>perfil-lipidico</t>
+          <t>calcio</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -905,12 +909,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2019-12-24_labs_quest-mx_tiroideo.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2019/labs/2019-12-24_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019/labs/2019-06-02_labs_quest-mx_calcio.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -918,22 +922,26 @@
           <t>move</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2019-06-02_labs_quest-mx_general.pdf') — '2/06/2019' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1qiH2_frLbKJ2vF2j6ICW6j9SRmbxxGU0/view</t>
+          <t>https://drive.google.com/file/d/1ffwqecdhzalYlS6o1XRwtznJRSrJ-KGV/view</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2020-04-17_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019-09-13_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2020-04-17</t>
+          <t>2019-09-13</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -943,22 +951,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>perfil-lipidico</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2020-04-17_labs_quest-mx_tiroideo.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2019-09-13_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2020/labs/2020-04-17_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -969,19 +977,19 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1pdBluP-dzl_wE0f_FWKaNH-l1mFrxZvw/view</t>
+          <t>https://drive.google.com/file/d/1txD2M8pAnAInDxjvL3pi712wRwmPTsPT/view</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2020-04-28_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019-12-24_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2020-04-28</t>
+          <t>2019-12-24</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -996,17 +1004,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2020-04-28_labs_quest-mx_tiroideo.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2019-12-24_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2020/labs/2020-04-28_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2019/labs/2019-12-24_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1017,19 +1025,19 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1JIAoEhyttwxc6Cv_SHEYfi9jodXjI9R7/view</t>
+          <t>https://drive.google.com/file/d/1qiH2_frLbKJ2vF2j6ICW6j9SRmbxxGU0/view</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020-04-17_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2020-05-25</t>
+          <t>2020-04-17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1039,7 +1047,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>perfil-lipidico</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1049,12 +1057,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2020-05-25_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2020-04-17_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020/labs/2020-04-17_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1065,19 +1073,19 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1sNLAT_auII9ux0kE0dNzDNi-5cmWi4H_/view</t>
+          <t>https://drive.google.com/file/d/1pdBluP-dzl_wE0f_FWKaNH-l1mFrxZvw/view</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2020-06-15_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020-04-28_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2020-06-15</t>
+          <t>2020-04-28</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1087,7 +1095,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-lipidico</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1097,12 +1105,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2020-06-15_labs_quest-mx_tiroglobulina.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2020-04-28_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2020/labs/2020-06-15_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/labs/2020-04-28_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1113,19 +1121,19 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1xq4z67ZNSeS-Ir5m3rtl17ElitnuZ2j4/view</t>
+          <t>https://drive.google.com/file/d/1JIAoEhyttwxc6Cv_SHEYfi9jodXjI9R7/view</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2021-12-22_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2021-12-22</t>
+          <t>2020-05-25</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1135,22 +1143,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>perfil-lipidico</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2021-12-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2020-05-25_labs_quest-mx_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2021/labs/2021-12-22_labs_quest-mx_perfil-lipidico.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1161,44 +1169,44 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1biQ7aNiS2p3mTi15rbgT2OE1HBr6scUP/view</t>
+          <t>https://drive.google.com/file/d/1sNLAT_auII9ux0kE0dNzDNi-5cmWi4H_/view</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025-08-11_labs_labcorp_general.pdf</t>
+          <t>2020-06-15_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2025-08-11</t>
+          <t>2020-06-15</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>labcorp</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2020-06-15_labs_quest-mx_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2025/labs/2025-08-11_labs_labcorp_general.pdf</t>
+          <t>2020/labs/2020-06-15_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1209,44 +1217,44 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1HMHksW_l3aF1lq9X3I0T0aSvDNNx3gpu/view</t>
+          <t>https://drive.google.com/file/d/1xq4z67ZNSeS-Ir5m3rtl17ElitnuZ2j4/view</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2020-12-10_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2020-12-10</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>labcorp</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>tiroglobulina</t>
+          <t>perfil-lipidico</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2020/labs/2020-12-10_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1254,47 +1262,51 @@
           <t>move</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf') — '10/12/2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
+          <t>https://drive.google.com/file/d/1kkEH36xcggv0M0nYPQP1z7GX8a6d1Q-3/view</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2021-06-07_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2021-06-07</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>labcorp</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>biometria</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2021/labs/2021-06-07_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1302,22 +1314,26 @@
           <t>move</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2021-06-07_labs_quest-mx_biometria.pdf') — '07/06/2021 9:49 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+          <t>https://drive.google.com/file/d/1CASli8xRI7Y1wLKR6oLBZ3JQRf-Y1KdU/view</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-17_labs_quest-mx_general.pdf</t>
+          <t>2021-12-22_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2021-12-22</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1327,22 +1343,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>perfil-lipidico</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2026-04-17_labs_quest-mx_biometria.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2021-12-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026/labs/2026-04-17_labs_quest-mx_general.pdf</t>
+          <t>2021/labs/2021-12-22_labs_quest-mx_perfil-lipidico.pdf</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1352,6 +1368,302 @@
       </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1biQ7aNiS2p3mTi15rbgT2OE1HBr6scUP/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2024-08-10_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2024-08-10</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>biometria</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-08-11_labs_labcorp_general.pdf</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2025-08-11</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>labcorp</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-08-11_labs_labcorp_general.pdf</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1HMHksW_l3aF1lq9X3I0T0aSvDNNx3gpu/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>labcorp</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>tiroglobulina</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-10-23_labs_labcorp_general.pdf</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2025-10-23</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>labcorp</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-05_labs_hospital-angeles-lomas_general.pdf</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>hospital-angeles-lomas</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_general.pdf</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf') — '05/03/2026' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-17_labs_quest-mx_general.pdf</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2026-04-17_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026/labs/2026-04-17_labs_quest-mx_general.pdf</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1UFeodi51jpRW9wcmxggZwTnSBr6yz8Yn/view</t>
         </is>
@@ -1368,7 +1680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -1438,22 +1750,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2019-03-11_radiologia_hospital-san-angel-inn_rastreo-yodo.pdf</t>
+          <t>2019-01-07_radiologia_hospital-angeles-pedregal_pet.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2019-03-11</t>
+          <t>2019-01-07</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>hospital-san-angel-inn</t>
+          <t>hospital-angeles-pedregal</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>rastreo-yodo</t>
+          <t>pet</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1463,12 +1775,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2019-03-11_nuclear_rastreo-yodo.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2019/radiologia/2019-03-11_radiologia_hospital-san-angel-inn_rastreo-yodo.pdf</t>
+          <t>2019/radiologia/2019-01-07_radiologia_hospital-angeles-pedregal_pet.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1476,27 +1788,31 @@
           <t>move</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf') — '07/01/2019' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1aia7BfJ-fw8149Vg-5iKgJZJ7g2IHK8l/view</t>
+          <t>https://drive.google.com/file/d/17PCU-FXw71gWbY5q8Id6_YjqM-d_BoVz/view</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2020-07-14_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+          <t>2019-03-11_radiologia_hospital-san-angel-inn_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2020-07-14</t>
+          <t>2019-03-11</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>hospital-angeles-pedregal</t>
+          <t>hospital-san-angel-inn</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1506,17 +1822,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2020</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2020-07-14_nuclear_rastreo-yodo.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2019-03-11_nuclear_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2020/radiologia/2020-07-14_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+          <t>2019/radiologia/2019-03-11_radiologia_hospital-san-angel-inn_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1527,44 +1843,44 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1rf96g6MjMv984xtt0QyWjjnklULtvj3N/view</t>
+          <t>https://drive.google.com/file/d/1aia7BfJ-fw8149Vg-5iKgJZJ7g2IHK8l/view</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2023-07-14_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+          <t>2019-08-21_radiologia_quest-mx_torax.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2023-07-14</t>
+          <t>2019-08-21</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>hospital-angeles-pedregal</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>pet</t>
+          <t>torax</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2023</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2019-08-21_rx_torax.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2023/radiologia/2023-07-14_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+          <t>2019/radiologia/2019-08-21_radiologia_quest-mx_torax.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1575,59 +1891,259 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FXbHPyQbqDHJOUMxnHiX_PjAFxFZ-3tH/view</t>
+          <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>2020-06-02_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2020-06-02</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2020/radiologia/2020-06-02_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf') — '02/06/2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1GcHOu5s7I3sn3A91BaqbSp0DkbtRu3tU/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2020-07-14_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2020-07-14</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>rastreo-yodo</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2020-07-14_nuclear_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2020/radiologia/2020-07-14_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1rf96g6MjMv984xtt0QyWjjnklULtvj3N/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2023-07-14_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2023-07-14</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>pet</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2023-07-14_pet_hospital-angeles-pedregal.pdf</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2023/radiologia/2023-07-14_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1FXbHPyQbqDHJOUMxnHiX_PjAFxFZ-3tH/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>2024-08-12_radiologia_hospital-angeles-pedregal_pet.pdf</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>2024-08-12</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>hospital-angeles-pedregal</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>pet</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>2026/ultrasonidos/REVISAR_2024-08-12_pet_hospital-angeles-pedregal.pdf</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>2024/radiologia/2024-08-12_radiologia_hospital-angeles-pedregal_pet.pdf</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>move</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>date order inferred from 2nd date on same document ('13/08/2024', unambiguous as DM) — '12/08/2024' itself was ambiguous</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/16xaHpUoMTXS17zDuCR9TG4nWF5YyvVkU/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-06_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>rastreo-yodo</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026/radiologia/2026-03-06_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf') — '06/03/2026' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1XEJc1QCLZ_7qVoTuM_paOCfx8BblEA1e/view</t>
         </is>
       </c>
     </row>
@@ -1647,7 +2163,7 @@
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
@@ -2004,7 +2520,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2014,7 +2530,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>hospital-angeles-lomas</t>
+          <t>hospital-angeles-pedregal</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2034,7 +2550,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2186,18 +2702,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
     <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -2256,7 +2772,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2266,7 +2782,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>hugo-dominguez-malagon</t>
+          <t>dominguez-malagon-patologia</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2286,7 +2802,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2304,48 +2820,152 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>2019-01-09_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2019-01-09</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>biopsia-tiroides</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2019/patologia/2019-01-09_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2019-01-09_patologia_diseccion-cuello.pdf') — '09-01-19' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1LYjog3waD7Oso0nAvtdOUpNEqfwYTmgY/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>2019-04-29</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>hospital-angeles-pedregal</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>mutacion-braf</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>2026/ultrasonidos/REVISAR_2019-04-29_patologia_braf-v600e.pdf</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>move</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr">
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1J4gLdlbUkRGF_aKpx6xqt-qvIimskL5x/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2020-06-05</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>hospital-angeles-pedregal</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>biopsia-tiroides</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf') — '05-06-2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1rRgSwtQWA6h02p8yGoUlgmc6Qc3x6DsU/view</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2430,7 +3050,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
+          <t>REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -2439,12 +3059,12 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-01-07_pet_hospital-angeles-pedregal.pdf</t>
+          <t>_REVISAR/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2454,19 +3074,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month — as printed ('07/01/2019') this is either 2019-01-07 (day-first) or 2019-07-01 (month-first); open the file to see which</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/17PCU-FXw71gWbY5q8Id6_YjqM-d_BoVz/view</t>
+          <t>https://drive.google.com/file/d/19PXsFTn8Hf3QyTUKLZGk5MDFmI978hn4/view</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
+          <t>REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -2475,12 +3095,12 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-01-09_patologia_diseccion-cuello.pdf</t>
+          <t>_REVISAR/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -2490,19 +3110,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month — as printed ('09-01-19') this is either 2019-01-09 (day-first) or 2019-09-01 (month-first); open the file to see which</t>
+          <t>date: ambiguous_day_month — as printed ('03/09/2022') this is either 2022-09-03 (day-first) or 2022-03-09 (month-first); open the file to see which (note: current filename implies 2022-10-03, which matches NEITHER reading — worth a closer look)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1LYjog3waD7Oso0nAvtdOUpNEqfwYTmgY/view</t>
+          <t>https://drive.google.com/file/d/1UECfx-gSSTtlJVsvrEzkGi6uh5okeiN-/view</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
+          <t>REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -2511,12 +3131,12 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-04-12_labs_quest-mx_tiroideo.pdf</t>
+          <t>_REVISAR/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -2526,19 +3146,19 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month — as printed ('4/12/2019') this is either 2019-12-04 (day-first) or 2019-04-12 (month-first); open the file to see which</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/10k9PIQTuP00FjD3--JFilIztJsAHzLex/view</t>
+          <t>https://drive.google.com/file/d/1yCWX0hgZnqKA57F22HZispDTzJKYOazt/view</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
+          <t>REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -2547,12 +3167,12 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-06-02_labs_quest-mx_general.pdf</t>
+          <t>_REVISAR/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -2562,19 +3182,19 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month — as printed ('2/06/2019') this is either 2019-06-02 (day-first) or 2019-02-06 (month-first); open the file to see which</t>
+          <t>date: no_date_found</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1ffwqecdhzalYlS6o1XRwtznJRSrJ-KGV/view</t>
+          <t>https://drive.google.com/file/d/1TCe5Bw2AmGt-EY4LEgt1cNaiWg-RwFLC/view</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>REVISAR_2019-08-21_rx_torax.pdf</t>
+          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr"/>
@@ -2583,12 +3203,12 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2019-08-21_rx_torax.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2019-08-21_rx_torax.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2598,532 +3218,116 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>date: no_date_found</t>
+          <t>date: ambiguous_day_month — as printed ('05/03/2026') this is either 2026-03-05 (day-first) or 2026-05-03 (month-first); open the file to see which (note: current filename implies 2026-03-06, which matches NEITHER reading — worth a closer look)</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
+          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
+          <t>DUP_2019-03-22_labs_quest-mx_tiroglobulina_2.pdf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2019-03-22</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>tiroglobulina</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
+          <t>2026/ultrasonidos/2019-03-22_labs_quest-mx_tiroglobulina_2.pdf</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
+          <t>_REVISAR/DUP_2019-03-22_labs_quest-mx_tiroglobulina_2.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>quarantine</t>
+          <t>duplicate</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>date: unparseable_date_text</t>
+          <t>duplicate of 2026/ultrasonidos/REVISAR_2019-03-22_labs_quest-mx_tiroglobulina.pdf (identical content hash)</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/19PXsFTn8Hf3QyTUKLZGk5MDFmI978hn4/view</t>
+          <t>https://drive.google.com/file/d/1sYDqEfhV3S73mf8WsjeDftvfe2gXcztV/view</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+          <t>DUP_REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2021-06-07</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>biometria</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-06-02_pet_hospital-angeles-pedregal.pdf</t>
+          <t>_REVISAR/DUP_REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>quarantine</t>
+          <t>duplicate</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month — as printed ('02/06/2020') this is either 2020-06-02 (day-first) or 2020-02-06 (month-first); open the file to see which</t>
+          <t>duplicate of 2026/ultrasonidos/REVISAR_2021-06-07_labs_quest-mx_biometria.pdf (identical content hash)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1GcHOu5s7I3sn3A91BaqbSp0DkbtRu3tU/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('05-06-2020') this is either 2020-06-05 (day-first) or 2020-05-06 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1rRgSwtQWA6h02p8yGoUlgmc6Qc3x6DsU/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2020-12-10_labs_quest-mx_tiroideo.pdf</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('10/12/2020') this is either 2020-12-10 (day-first) or 2020-10-12 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1kkEH36xcggv0M0nYPQP1z7GX8a6d1Q-3/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2021-06-07_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('07/06/2021 9:49 AM') this is either 2021-06-07 (day-first) or 2021-07-06 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1CASli8xRI7Y1wLKR6oLBZ3JQRf-Y1KdU/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('07/06/2021 9:49 AM') this is either 2021-06-07 (day-first) or 2021-07-06 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
           <t>https://drive.google.com/file/d/1nuqeeVhX0deJ7BwXzsKAfsUsOPgi_HLF/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('03/09/2022') this is either 2022-09-03 (day-first) or 2022-03-09 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1UECfx-gSSTtlJVsvrEzkGi6uh5okeiN-/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>date: no_date_found</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1yCWX0hgZnqKA57F22HZispDTzJKYOazt/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>date: no_date_found</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1TCe5Bw2AmGt-EY4LEgt1cNaiWg-RwFLC/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('10/08/2024 9:38 AM') this is either 2024-08-10 (day-first) or 2024-10-08 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('05/03/2026') this is either 2026-03-05 (day-first) or 2026-05-03 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('05/03/2026') this is either 2026-03-05 (day-first) or 2026-05-03 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-06_pet_hospital-angeles-pedregal.pdf</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('06/03/2026') this is either 2026-03-06 (day-first) or 2026-06-03 (month-first); open the file to see which</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1XEJc1QCLZ_7qVoTuM_paOCfx8BblEA1e/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>DUP_2019-03-22_labs_quest-mx_tiroglobulina_2.pdf</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>2019-03-22</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>quest-mx</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>tiroglobulina</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/2019-03-22_labs_quest-mx_tiroglobulina_2.pdf</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>_REVISAR/DUP_2019-03-22_labs_quest-mx_tiroglobulina_2.pdf</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>duplicate</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>duplicate of 2026/ultrasonidos/REVISAR_2019-03-22_labs_quest-mx_tiroglobulina.pdf (identical content hash)</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1sYDqEfhV3S73mf8WsjeDftvfe2gXcztV/view</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update master tracker 2026-08-29 16:04 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29 15:47</t>
+          <t>2026-08-29 16:04</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -556,7 +556,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -570,7 +570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -1376,12 +1376,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2024-08-10_labs_quest-mx_biometria.pdf</t>
+          <t>2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2024-08-10</t>
+          <t>2022-11-22</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1391,22 +1391,22 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>biometria</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1416,49 +1416,49 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('REVISAR_2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
+          <t>https://drive.google.com/file/d/1yCWX0hgZnqKA57F22HZispDTzJKYOazt/view</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-08-11_labs_labcorp_general.pdf</t>
+          <t>2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2025-08-11</t>
+          <t>2023-07-12</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>labcorp</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>biometria</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2025/labs/2025-08-11_labs_labcorp_general.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1466,47 +1466,51 @@
           <t>move</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('REVISAR_2023-07-12_labs_quest-mx_biometria.pdf') already matches the day-first reading.</t>
+        </is>
+      </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1HMHksW_l3aF1lq9X3I0T0aSvDNNx3gpu/view</t>
+          <t>https://drive.google.com/file/d/1TCe5Bw2AmGt-EY4LEgt1cNaiWg-RwFLC/view</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2024-08-10</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>labcorp</t>
+          <t>quest-mx</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>tiroglobulina</t>
+          <t>biometria</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2024/labs/2024-08-10_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1514,22 +1518,26 @@
           <t>move</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024 9:38 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
+          <t>https://drive.google.com/file/d/1U5k59WV7Nm3fxTR-RdoFkBc2Ka9MUi6U/view</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025-08-11_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2025-10-23</t>
+          <t>2025-08-11</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1549,12 +1557,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2025-08-11_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025/labs/2025-08-11_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1565,44 +1573,44 @@
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+          <t>https://drive.google.com/file/d/1HMHksW_l3aF1lq9X3I0T0aSvDNNx3gpu/view</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-03-05_labs_hospital-angeles-lomas_general.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-03-05</t>
+          <t>2025-10-23</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>hospital-angeles-lomas</t>
+          <t>labcorp</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>tiroglobulina</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2025-08-30_labs_labcorp-ny_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_general.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1610,51 +1618,47 @@
           <t>move</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>date confirmed via existing filename ('REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf') — '05/03/2026' was ambiguous on its own, but the current name already matches the day-first reading</t>
-        </is>
-      </c>
+      <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
+          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-04-17_labs_quest-mx_general.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2025-10-23</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>quest-mx</t>
+          <t>labcorp</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2026-04-17_labs_quest-mx_biometria.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2025-10-24_labs_labcorp-ny_general.pdf</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026/labs/2026-04-17_labs_quest-mx_general.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1664,6 +1668,106 @@
       </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-05_labs_hospital-angeles-lomas_general.pdf</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>hospital-angeles-lomas</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026/labs/2026-03-05_labs_hospital-angeles-lomas_general.pdf</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>date confirmed via existing filename ('REVISAR_2026-03-05_labs_hospital-angeles-lomas_biometria.pdf') — '05/03/2026' was ambiguous on its own, but the current name already matches the day-first reading</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1hwKjPws8DSHIvD5n-7AkVqLdbvp1Usjk/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-04-17_labs_quest-mx_general.pdf</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-04-17</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2026-04-17_labs_quest-mx_biometria.pdf</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026/labs/2026-04-17_labs_quest-mx_general.pdf</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1UFeodi51jpRW9wcmxggZwTnSBr6yz8Yn/view</t>
         </is>
@@ -2163,7 +2267,7 @@
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
@@ -2472,7 +2576,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
+          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2487,7 +2591,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ultrasonido-cuello</t>
+          <t>ultrasonido-tiroides</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2502,7 +2606,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2520,7 +2624,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2530,7 +2634,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>hospital-angeles-pedregal</t>
+          <t>hospital-angeles-lomas</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2550,7 +2654,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2702,13 +2806,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -2772,7 +2876,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dr-dominguez-malagon_inmunohistoquimica.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2782,12 +2886,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>dominguez-malagon-patologia</t>
+          <t>dr-dominguez-malagon</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>biopsia-tiroides</t>
+          <t>inmunohistoquimica</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -2802,7 +2906,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_inmunohistoquimica.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2920,50 +3024,102 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>2020-06-01_patologia_nucleo-diagnostico_biopsia-ganglio.pdf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2020-06-01</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>nucleo-diagnostico</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>biopsia-ganglio</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026/ultrasonidos/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_biopsia-ganglio.pdf</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de Reporte (encabezado del documento): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/19PXsFTn8Hf3QyTUKLZGk5MDFmI978hn4/view</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>2020-06-05</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>hospital-angeles-pedregal</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>biopsia-tiroides</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>2020</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>2026/ultrasonidos/REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>move</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>move</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>date confirmed via existing filename ('REVISAR_2020-06-05_patologia_ganglios-cervicales.pdf') — '05-06-2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1rRgSwtQWA6h02p8yGoUlgmc6Qc3x6DsU/view</t>
         </is>
@@ -2980,7 +3136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -3050,7 +3206,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
+          <t>REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr"/>
@@ -3059,12 +3215,12 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2020-06-01_patologia_baaf-ganglio.pdf</t>
+          <t>_REVISAR/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -3074,19 +3230,19 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date: no_date_found</t>
+          <t>date: ambiguous_day_month — as printed ('03/09/2022') this is either 2022-09-03 (day-first) or 2022-03-09 (month-first); open the file to see which (note: current filename implies 2022-10-03, which matches NEITHER reading — worth a closer look)</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/19PXsFTn8Hf3QyTUKLZGk5MDFmI978hn4/view</t>
+          <t>https://drive.google.com/file/d/1UECfx-gSSTtlJVsvrEzkGi6uh5okeiN-/view</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -3095,12 +3251,12 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2022-10-03_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -3110,222 +3266,114 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>date: ambiguous_day_month — as printed ('03/09/2022') this is either 2022-09-03 (day-first) or 2022-03-09 (month-first); open the file to see which (note: current filename implies 2022-10-03, which matches NEITHER reading — worth a closer look)</t>
+          <t>date: ambiguous_day_month — as printed ('05/03/2026') this is either 2026-03-05 (day-first) or 2026-05-03 (month-first); open the file to see which (note: current filename implies 2026-03-06, which matches NEITHER reading — worth a closer look)</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1UECfx-gSSTtlJVsvrEzkGi6uh5okeiN-/view</t>
+          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+          <t>DUP_2019-03-22_labs_quest-mx_tiroglobulina_2.pdf</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2019-03-22</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>tiroglobulina</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
+          <t>2026/ultrasonidos/2019-03-22_labs_quest-mx_tiroglobulina_2.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2022-11-22_labs_quest-mx_tiroglobulina-estimulada.pdf</t>
+          <t>_REVISAR/DUP_2019-03-22_labs_quest-mx_tiroglobulina_2.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>quarantine</t>
+          <t>duplicate</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>date: no_date_found</t>
+          <t>duplicate of 2026/ultrasonidos/REVISAR_2019-03-22_labs_quest-mx_tiroglobulina.pdf (identical content hash)</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1yCWX0hgZnqKA57F22HZispDTzJKYOazt/view</t>
+          <t>https://drive.google.com/file/d/1sYDqEfhV3S73mf8WsjeDftvfe2gXcztV/view</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
+          <t>DUP_REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2021-06-07</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>quest-mx</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>biometria</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>2026/ultrasonidos/REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>_REVISAR/REVISAR_2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>_REVISAR/DUP_REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>quarantine</t>
+          <t>duplicate</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>date: no_date_found</t>
+          <t>duplicate of 2026/ultrasonidos/REVISAR_2021-06-07_labs_quest-mx_biometria.pdf (identical content hash)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1TCe5Bw2AmGt-EY4LEgt1cNaiWg-RwFLC/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>_REVISAR/REVISAR_2026-03-06_labs_hospital-angeles-lomas_biometria.pdf</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>quarantine</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>date: ambiguous_day_month — as printed ('05/03/2026') this is either 2026-03-05 (day-first) or 2026-05-03 (month-first); open the file to see which (note: current filename implies 2026-03-06, which matches NEITHER reading — worth a closer look)</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1q6YfszsnBRSFzts8znV0Pk7NgcllqlyB/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>DUP_2019-03-22_labs_quest-mx_tiroglobulina_2.pdf</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>2019-03-22</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>quest-mx</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>tiroglobulina</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/2019-03-22_labs_quest-mx_tiroglobulina_2.pdf</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>_REVISAR/DUP_2019-03-22_labs_quest-mx_tiroglobulina_2.pdf</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>duplicate</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>duplicate of 2026/ultrasonidos/REVISAR_2019-03-22_labs_quest-mx_tiroglobulina.pdf (identical content hash)</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/file/d/1sYDqEfhV3S73mf8WsjeDftvfe2gXcztV/view</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>DUP_REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>2021-06-07</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>quest-mx</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>biometria</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>_REVISAR/DUP_REVISAR_2021-06-07_labs_quest-mx_biometria_2.pdf</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>duplicate</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>duplicate of 2026/ultrasonidos/REVISAR_2021-06-07_labs_quest-mx_biometria.pdf (identical content hash)</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1nuqeeVhX0deJ7BwXzsKAfsUsOPgi_HLF/view</t>
         </is>

</xml_diff>

<commit_message>
chore: update master tracker 2026-08-29 16:16 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -461,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29 16:04</t>
+          <t>2026-08-29 16:16</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>dry run (plan only, nothing changed on Drive)</t>
+          <t>apply (changes executed)</t>
         </is>
       </c>
     </row>
@@ -576,7 +576,7 @@
     <col width="52" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -836,7 +836,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019-05-15_labs_quest-mx_general-orina.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -851,7 +851,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>general-orina</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1376,7 +1376,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1406,7 +1406,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1428,7 +1428,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>biometria</t>
+          <t>biometria-hematica</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('REVISAR_2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024 9:38 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('REVISAR_2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1628,7 +1628,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025-10-23_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1643,7 +1643,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>general</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1992,7 +1992,11 @@
           <t>move</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de Reporte (encabezado): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
@@ -2576,7 +2580,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
+          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2591,7 +2595,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>ultrasonido-tiroides</t>
+          <t>ultrasonido-cuello</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -2606,7 +2610,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2812,7 +2816,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -2876,7 +2880,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_dr-dominguez-malagon_inmunohistoquimica.pdf</t>
+          <t>2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2886,12 +2890,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>dr-dominguez-malagon</t>
+          <t>dr-hugo-dominguez-malagon</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>inmunohistoquimica</t>
+          <t>biopsia-tiroides</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -2906,7 +2910,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_inmunohistoquimica.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -3024,7 +3028,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2020-06-01_patologia_nucleo-diagnostico_biopsia-ganglio.pdf</t>
+          <t>2020-06-01_patologia_nucleo-diagnostico_citologia-baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3039,7 +3043,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>biopsia-ganglio</t>
+          <t>citologia-baaf-ganglio</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -3054,7 +3058,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_biopsia-ganglio.pdf</t>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -3064,7 +3068,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de Reporte (encabezado del documento): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha del reporte (encabezado, Ciudad de México): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">

</xml_diff>

<commit_message>
chore: update master tracker 2026-08-29 18:19 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29 16:52</t>
+          <t>2026-08-29 18:19</t>
         </is>
       </c>
     </row>
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6">
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -682,7 +682,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -794,7 +794,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>dominguez-malagon</t>
+          <t>hugo-dominguez-malagon</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -850,19 +850,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -914,6 +914,38 @@
       <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Drive Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>master_tracker.xlsx</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>master_tracker.xlsx</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>ignored</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>unsupported file type (application/vnd.openxmlformats-officedocument.spreadsheetml.sheet) — left alone</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://drive.google.com/file/d/1VgiaxWywpKl0pfX7z1szCbbyMzcDeGhn/view</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1456,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025-10-23_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1444,7 +1476,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>general</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1454,12 +1486,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -2158,7 +2190,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2178,7 +2210,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2188,12 +2220,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -2706,7 +2738,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2020-06-01_patologia_nucleo-diagnostico_biopsia-ganglio.pdf</t>
+          <t>2020-06-01_patologia_nucleo-diagnostico_citologia-ganglio.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2726,7 +2758,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>biopsia-ganglio</t>
+          <t>citologia-ganglio</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2736,7 +2768,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_biopsia-ganglio.pdf</t>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-ganglio.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2746,7 +2778,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha del reporte (encabezado, Ciudad de México, a...): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha del reporte (Ciudad de México, a...): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -2810,7 +2842,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglionar.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2830,7 +2862,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>biopsia-tiroides</t>
+          <t>biopsia-ganglionar</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2840,12 +2872,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglionar.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -3576,7 +3608,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de Reporte: '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha del reporte (encabezado): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">

</xml_diff>

<commit_message>
chore: update master tracker 2026-08-29 18:28 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29 18:19</t>
+          <t>2026-08-29 18:28</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>dry run (plan only, nothing changed on Drive)</t>
+          <t>apply (changes executed)</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -794,7 +794,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -809,7 +809,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>hugo-dominguez-malagon</t>
+          <t>dr-dominguez-malagon</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -824,7 +824,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1134,7 +1134,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-06_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+          <t>2026-03-06_radiologia_hospital-angeles-pedregal_pet.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1154,7 +1154,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>rastreo-yodo</t>
+          <t>pet</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1164,12 +1164,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026/radiologia/2026-03-06_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
+          <t>2026/radiologia/2026-03-06_radiologia_hospital-angeles-pedregal_pet.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1749,7 +1749,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023 8:20 AM'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria-hematica.pdf') already matches the day-first reading.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria-hematica.pdf') already matches the day-first reading.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1912,7 +1912,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
+          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1932,7 +1932,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ultrasonido-cuello</t>
+          <t>ultrasonido-tiroides</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1942,12 +1942,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -2190,7 +2190,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2022-11-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2220,12 +2220,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -2778,7 +2778,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha del reporte (Ciudad de México, a...): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Ciudad de México, a (fecha de reporte): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -2842,7 +2842,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglionar.pdf</t>
+          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2862,7 +2862,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>biopsia-ganglionar</t>
+          <t>biopsia-tiroides</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2872,12 +2872,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglionar.pdf</t>
+          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -3030,7 +3030,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_perfil-lipidico.pdf') — '10/12/2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_perfil-lipidico.pdf') — '10/12/2020 9:08 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -3468,7 +3468,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019-05-15_labs_quest-mx_general-orina.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3488,7 +3488,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>general-orina</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -3498,12 +3498,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -3606,11 +3606,7 @@
           <t>no_change</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha del reporte (encabezado): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
-        </is>
-      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>

</xml_diff>

<commit_message>
chore: update master tracker 2026-08-30 12:45 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29 18:28</t>
+          <t>2026-08-30 12:45</t>
         </is>
       </c>
     </row>
@@ -604,64 +604,76 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>This script never guesses on an unclear date or category — anything it can't confidently resolve (even after checking its current folder as a fallback) gets moved into Medical/_REVISAR, prefixed REVISAR_. Duplicates land there too, prefixed DUP_. This runs automatically every night, so _REVISAR is the daily check: review what's in there and move each file to where it belongs by hand.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Category (all years)</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Files</t>
         </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>labs</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>radiologia</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ultrasonidos</t>
+          <t>labs</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>7</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>inbody</t>
+          <t>radiologia</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>ultrasonidos</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>inbody</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>patologia</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B25" t="n">
         <v>5</v>
       </c>
     </row>
@@ -682,7 +694,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -794,7 +806,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -809,7 +821,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>dr-dominguez-malagon</t>
+          <t>dr-hugo-dominguez-malagon</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -819,12 +831,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>2018/patologia/2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1134,7 +1146,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-03-06_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+          <t>2026-03-06_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1154,19 +1166,19 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>pet</t>
+          <t>rastreo-yodo</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>2026/radiologia/2026-03-06_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>2026/radiologia/2026-03-06_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026/radiologia/2026-03-06_radiologia_hospital-angeles-pedregal_pet.pdf</t>
-        </is>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>rename</t>
@@ -1174,7 +1186,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2026-03-06_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf') — '06/03/2026' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2026-03-06_radiologia_hospital-angeles-pedregal_pet.pdf') — '06/03/2026' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1186,7 +1198,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1201,7 +1213,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>hospital-angeles-lomas</t>
+          <t>hospital-angeles-pedregal</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1216,12 +1228,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -1670,7 +1682,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024 9:38 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1749,7 +1761,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -1837,7 +1849,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1847,12 +1859,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria-hematica.pdf') already matches the day-first reading.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria.pdf') already matches the day-first reading.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1912,7 +1924,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
+          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1932,17 +1944,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ultrasonido-tiroides</t>
+          <t>ultrasonido-cuello</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -2063,7 +2075,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>2022/labs/2022-03-09_labs_quest-usa_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2073,12 +2085,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroglobulina.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
+          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroideo.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2190,7 +2202,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2210,17 +2222,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -2738,7 +2750,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2020-06-01_patologia_nucleo-diagnostico_citologia-ganglio.pdf</t>
+          <t>2020-06-01_patologia_nucleo-diagnostico_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2758,17 +2770,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>citologia-ganglio</t>
+          <t>baaf-ganglio</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-baaf-ganglio.pdf</t>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-ganglio.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-ganglio.pdf</t>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2778,7 +2790,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Ciudad de México, a (fecha de reporte): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha del reporte (Ciudad de México, a...): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -3030,7 +3042,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_perfil-lipidico.pdf') — '10/12/2020 9:08 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_perfil-lipidico.pdf') — '10/12/2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -3057,7 +3069,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -3272,7 +3284,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2019-03-18_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019-03-18_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3292,7 +3304,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -3302,12 +3314,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2019/labs/2019-03-18_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/labs/2019-03-18_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -3468,7 +3480,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2019-05-15_labs_quest-mx_general-orina.pdf</t>
+          <t>2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3488,7 +3500,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>general-orina</t>
+          <t>general</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -3498,12 +3510,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -3664,7 +3676,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019-09-13_labs_quest-mx_perfil-tiroideo-lipidico.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3684,7 +3696,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo-lipidico</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -3694,12 +3706,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
+          <t>2019/labs/2019-09-13_labs_quest-mx_perfil-tiroideo-lipidico.pdf</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: update master tracker 2026-08-31 15:02 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-30 12:45</t>
+          <t>2026-08-31 15:02</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026/radiologia/2026-03-06_radiologia_hospital-angeles-pedregal_pet.pdf</t>
+          <t>2026/radiologia/2026-03-06_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1181,12 +1181,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2026-03-06_radiologia_hospital-angeles-pedregal_pet.pdf') — '06/03/2026' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2026-03-06_radiologia_hospital-angeles-pedregal_rastreo-yodo.pdf') — '06/03/2026' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>hospital-angeles-pedregal</t>
+          <t>hospital-angeles-lomas</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -2227,7 +2227,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2021-06-07_labs_quest-mx_biometria.pdf') — '07/06/2021 9:49 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2021-06-07_labs_quest-mx_biometria.pdf') — '07/06/2021' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2495,7 +2495,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -2654,7 +2654,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2020-05-23_ultrasonidos_otro_ultrasonido-tiroides.pdf</t>
+          <t>2020-05-23_ultrasonidos_otro_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ultrasonido-tiroides</t>
+          <t>ultrasonido-cuello</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -2684,12 +2684,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2020/ultrasonidos/2020-05-23_ultrasonidos_otro_ultrasonido-tiroides.pdf</t>
+          <t>2020/ultrasonidos/2020-05-23_ultrasonidos_otro_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -2750,7 +2750,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2020-06-01_patologia_nucleo-diagnostico_baaf-ganglio.pdf</t>
+          <t>2020-06-01_patologia_nucleo-diagnostico_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2770,17 +2770,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>baaf-ganglio</t>
+          <t>biopsia-tiroides</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-ganglio.pdf</t>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_baaf-ganglio.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_baaf-ganglio.pdf</t>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2788,11 +2788,7 @@
           <t>rename</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha del reporte (Ciudad de México, a...): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
-        </is>
-      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/19PXsFTn8Hf3QyTUKLZGk5MDFmI978hn4/view</t>
@@ -3069,7 +3065,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -3284,7 +3280,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2019-03-18_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2019-03-18_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3304,17 +3300,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>2019/labs/2019-03-18_labs_quest-mx_perfil-tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>2019/labs/2019-03-18_labs_quest-mx_tiroideo.pdf</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2019/labs/2019-03-18_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -3480,7 +3476,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019-05-15_labs_quest-mx_examen-general-orina.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3500,17 +3496,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>examen-general-orina</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_examen-general-orina.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -3618,7 +3614,11 @@
           <t>no_change</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de reporte (encabezado): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
@@ -3676,7 +3676,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2019-09-13_labs_quest-mx_perfil-tiroideo-lipidico.pdf</t>
+          <t>2019-09-13_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3696,17 +3696,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>perfil-tiroideo-lipidico</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>2019/labs/2019-09-13_labs_quest-mx_perfil-tiroideo-lipidico.pdf</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>2019/labs/2019-09-13_labs_quest-mx_perfil-tiroideo-lipidico.pdf</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">

</xml_diff>

<commit_message>
chore: update master tracker 2026-09-01 12:32 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-31 15:02</t>
+          <t>2026-09-01 12:32</t>
         </is>
       </c>
     </row>
@@ -1198,7 +1198,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>hospital-angeles-lomas</t>
+          <t>hospital-angeles-pedregal</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1468,7 +1468,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1498,12 +1498,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -1824,7 +1824,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>biometria</t>
+          <t>biometria-hematica</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1854,12 +1854,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -2050,7 +2050,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2022-03-09_labs_quest-usa_tiroideo.pdf</t>
+          <t>2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>tiroglobulina</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2080,12 +2080,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2022/labs/2022-03-09_labs_quest-usa_tiroideo.pdf</t>
+          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>date order inferred from 2nd date on same document ('5/20/2020', unambiguous as MD) — '3/10/2022' itself was ambiguous</t>
+          <t>date confirmed via existing filename ('2022-03-10_ultrasonidos_envision-imaging_ultrasonido-tiroides.pdf') — '3/10/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -2202,7 +2202,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2022-11-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2232,17 +2232,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022 8:58 AM'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -2495,7 +2495,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -2654,7 +2654,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2020-05-23_ultrasonidos_otro_ultrasonido-cuello.pdf</t>
+          <t>2020-05-23_ultrasonidos_otro_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2674,17 +2674,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ultrasonido-cuello</t>
+          <t>ultrasonido-tiroides</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>2020/ultrasonidos/2020-05-23_ultrasonidos_otro_ultrasonido-cuello.pdf</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>2020/ultrasonidos/2020-05-23_ultrasonidos_otro_ultrasonido-tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2020/ultrasonidos/2020-05-23_ultrasonidos_otro_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_baaf-ganglio.pdf</t>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2785,7 +2785,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_perfil-lipidico.pdf') — '10/12/2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_perfil-lipidico.pdf') — '10/12/2020 9:08 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -3065,7 +3065,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -3305,7 +3305,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2019/labs/2019-03-18_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2019/labs/2019-03-18_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -3476,7 +3476,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2019-05-15_labs_quest-mx_examen-general-orina.pdf</t>
+          <t>2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3496,17 +3496,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>examen-general-orina</t>
+          <t>general</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>2019/labs/2019-05-15_labs_quest-mx_examen-general-orina.pdf</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_examen-general-orina.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -3614,11 +3614,7 @@
           <t>no_change</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de reporte (encabezado): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
-        </is>
-      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>
@@ -3701,7 +3697,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2019/labs/2019-09-13_labs_quest-mx_perfil-tiroideo-lipidico.pdf</t>
+          <t>2019/labs/2019-09-13_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -3711,7 +3707,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: update master tracker 2026-09-02 12:06 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-01 12:32</t>
+          <t>2026-09-02 12:06</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -806,7 +806,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_hugo-ricardo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>dr-hugo-dominguez-malagon</t>
+          <t>hugo-ricardo-dominguez-malagon</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -836,12 +836,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_hugo-ricardo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -1198,7 +1198,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>hospital-angeles-pedregal</t>
+          <t>hospital-angeles</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1468,7 +1468,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1488,35 +1488,35 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>tiroglobulina</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025-10-23_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1536,28 +1536,28 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>tiroglobulina</t>
+          <t>general</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
+          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria.pdf') already matches the day-first reading.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023 8:20 AM'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria-hematica.pdf') already matches the day-first reading.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2050,7 +2050,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>2022-03-09_labs_quest-usa_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2070,19 +2070,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>tiroglobulina</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>2022/labs/2022-03-09_labs_quest-usa_tiroideo.pdf</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>rename</t>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroideo.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
+          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroglobulina.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2142,7 +2142,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2022-03-10_ultrasonidos_envision-imaging_ultrasonido-tiroides.pdf') — '3/10/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
+          <t>date order inferred from 2nd date on same document ('5/20/2020', unambiguous as MD) — '3/10/2022' itself was ambiguous</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -2202,7 +2202,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2222,19 +2222,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
-        </is>
-      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>rename</t>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022 8:58 AM'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2021-06-07_labs_quest-mx_biometria.pdf') — '07/06/2021' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2021-06-07_labs_quest-mx_biometria.pdf') — '07/06/2021 9:49 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2679,7 +2679,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2020/ultrasonidos/2020-05-23_ultrasonidos_otro_ultrasonido-cuello.pdf</t>
+          <t>2020/ultrasonidos/2020-05-23_ultrasonidos_otro_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -2702,7 +2702,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2732,12 +2732,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -2902,7 +2902,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2020-06-15_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020-06-15_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2932,12 +2932,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2020/labs/2020-06-15_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/labs/2020-06-15_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_perfil-lipidico.pdf') — '10/12/2020 9:08 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_perfil-lipidico.pdf') — '10/12/2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -3476,7 +3476,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019-05-15_labs_quest-mx_general-orina.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3496,17 +3496,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>general-orina</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_examen-general-orina.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">

</xml_diff>

<commit_message>
chore: update master tracker 2026-09-03 12:06 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-02 12:06</t>
+          <t>2026-09-03 12:06</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -806,7 +806,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_hugo-ricardo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_hospital-satelite_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>hugo-ricardo-dominguez-malagon</t>
+          <t>hospital-satelite</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_hugo-ricardo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_hugo-ricardo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_hospital-satelite_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -1468,7 +1468,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025-10-23_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1488,17 +1488,17 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>tiroglobulina</t>
+          <t>general</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1509,14 +1509,14 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
+          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1536,28 +1536,28 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>tiroglobulina</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024 9:38 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1761,7 +1761,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023 8:20 AM'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria-hematica.pdf') already matches the day-first reading.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria-hematica.pdf') already matches the day-first reading.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1924,7 +1924,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
+          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ultrasonido-cuello</t>
+          <t>ultrasonido-tiroides</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1954,12 +1954,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>2022/labs/2022-03-09_labs_quest-usa_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2085,12 +2085,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroglobulina.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
+          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroideo.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2202,7 +2202,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2022-11-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2222,19 +2222,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
-        </is>
-      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>rename</t>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022 8:58 AM'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -2902,7 +2902,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2020-06-15_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020-06-15_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2922,17 +2922,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>2020/labs/2020-06-15_labs_quest-mx_perfil-tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>2020/labs/2020-06-15_labs_quest-mx_tiroideo.pdf</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2020/labs/2020-06-15_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_perfil-lipidico.pdf') — '10/12/2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_perfil-lipidico.pdf') — '10/12/2020 9:08 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -3428,7 +3428,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
+          <t>2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>mutacion-braf</t>
+          <t>biopsia-tiroides</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -3458,12 +3458,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
+          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -3476,7 +3476,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2019-05-15_labs_quest-mx_general-orina.pdf</t>
+          <t>2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3496,17 +3496,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>general-orina</t>
+          <t>general</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">

</xml_diff>

<commit_message>
chore: update master tracker 2026-09-04 12:07 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-03 12:06</t>
+          <t>2026-09-04 12:07</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -806,7 +806,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_hospital-satelite_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>hospital-satelite</t>
+          <t>dr-dominguez-malagon</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_hugo-ricardo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_hospital-satelite_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_hospital-satelite_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024 9:38 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1761,7 +1761,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -1824,7 +1824,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
+          <t>2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>biometria-hematica</t>
+          <t>biometria</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1854,17 +1854,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria-hematica.pdf') already matches the day-first reading.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023 8:20 AM'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria-hematica.pdf') already matches the day-first reading.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1924,7 +1924,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
+          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1944,17 +1944,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ultrasonido-tiroides</t>
+          <t>ultrasonido-cuello</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -2050,7 +2050,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2022-03-09_labs_quest-usa_tiroideo.pdf</t>
+          <t>2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>tiroglobulina</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2080,12 +2080,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2022/labs/2022-03-09_labs_quest-usa_tiroideo.pdf</t>
+          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -2202,7 +2202,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2222,19 +2222,19 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
-        </is>
-      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>rename</t>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022 8:58 AM'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -2495,7 +2495,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -2702,7 +2702,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2732,12 +2732,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -2850,7 +2850,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglios-linfaticos.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>biopsia-tiroides</t>
+          <t>biopsia-ganglios-linfaticos</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2880,12 +2880,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglios-linfaticos.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2020/labs/2020-06-15_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020/labs/2020-06-15_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2937,7 +2937,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_perfil-lipidico.pdf') — '10/12/2020 9:08 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2020-12-10_labs_quest-mx_perfil-lipidico.pdf') — '10/12/2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
+          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -3463,7 +3463,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>

</xml_diff>

<commit_message>
chore: update master tracker 2026-09-05 11:17 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-04 12:07</t>
+          <t>2026-09-05 11:17</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -806,7 +806,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dr-dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>dr-dominguez-malagon</t>
+          <t>dr-dominguez-malagon-patologia</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_hospital-satelite_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>hospital-angeles</t>
+          <t>hospital-angeles-lomas</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1228,12 +1228,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023 8:20 AM'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria-hematica.pdf') already matches the day-first reading.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023 8:20 AM'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria.pdf') already matches the day-first reading.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2022/labs/2022-03-09_labs_quest-usa_tiroideo.pdf</t>
+          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2085,12 +2085,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroideo.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
+          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroglobulina.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -2495,7 +2495,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -2702,7 +2702,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2722,17 +2722,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -2850,7 +2850,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglios-linfaticos.pdf</t>
+          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2870,19 +2870,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>biopsia-ganglios-linfaticos</t>
+          <t>biopsia-tiroides</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
+          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglios-linfaticos.pdf</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
           <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglios-linfaticos.pdf</t>
-        </is>
-      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>rename</t>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf') — '05-06-2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglios-linfaticos.pdf') — '05-06-2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -3614,7 +3614,11 @@
           <t>no_change</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de reporte (encabezado, sin etiqueta explícita): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>

</xml_diff>

<commit_message>
chore: update master tracker 2026-09-06 11:39 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-05 11:17</t>
+          <t>2026-09-06 11:39</t>
         </is>
       </c>
     </row>
@@ -806,7 +806,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_dr-dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_hugo-ricardo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>dr-dominguez-malagon-patologia</t>
+          <t>hugo-ricardo-dominguez-malagon</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_hugo-ricardo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>hospital-angeles-lomas</t>
+          <t>hospital-angeles-pedregal</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1468,7 +1468,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1488,7 +1488,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1498,12 +1498,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024 9:38 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2050,7 +2050,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>2022-03-09_labs_quest-usa_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>tiroglobulina</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2080,12 +2080,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>2022/labs/2022-03-09_labs_quest-usa_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -2875,7 +2875,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglios-linfaticos.pdf</t>
+          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -2885,12 +2885,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglios-linfaticos.pdf') — '05-06-2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf') — '05-06-2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -3616,7 +3616,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de reporte (encabezado, sin etiqueta explícita): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha (sin etiqueta explícita, bajo el encabezado 'Laboratorios de Análisis Clínicos'): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">

</xml_diff>

<commit_message>
chore: update master tracker 2026-09-07 13:27 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-06 11:39</t>
+          <t>2026-09-07 13:27</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -806,7 +806,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_hugo-ricardo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>hugo-ricardo-dominguez-malagon</t>
+          <t>dominguez-malagon-patologia</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dr-dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_hugo-ricardo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_hugo-ricardo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -1468,7 +1468,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1488,35 +1488,35 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>tiroglobulina</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1536,17 +1536,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>tiroglobulina</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1557,7 +1557,7 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
+          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024 9:38 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>2022/labs/2022-03-09_labs_quest-usa_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2085,12 +2085,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroglobulina.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
+          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroideo.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2202,7 +2202,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2022-11-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2232,12 +2232,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -2702,7 +2702,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2732,12 +2732,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -3616,7 +3616,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha (sin etiqueta explícita, bajo el encabezado 'Laboratorios de Análisis Clínicos'): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de reporte (sin etiqueta explícita, encabezado del documento): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">

</xml_diff>

<commit_message>
chore: update master tracker 2026-09-08 12:08 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-07 13:27</t>
+          <t>2026-09-08 12:08</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -806,7 +806,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>dominguez-malagon-patologia</t>
+          <t>dr-hugo-dominguez-malagon</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_hugo-ricardo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>hospital-angeles-pedregal</t>
+          <t>hospital-angeles-lomas</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1228,12 +1228,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -1516,7 +1516,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025-10-23_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>general</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1546,12 +1546,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024 9:38 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1824,7 +1824,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>biometria</t>
+          <t>biometria-hematica</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1854,17 +1854,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023 8:20 AM'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria.pdf') already matches the day-first reading.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria.pdf') already matches the day-first reading.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -2727,7 +2727,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -3476,7 +3476,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019-05-15_labs_quest-mx_general-orina.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3496,7 +3496,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>general-orina</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -3506,12 +3506,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -3614,11 +3614,7 @@
           <t>no_change</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de reporte (sin etiqueta explícita, encabezado del documento): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
-        </is>
-      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>

</xml_diff>

<commit_message>
chore: update master tracker 2026-09-09 12:19 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-08 12:08</t>
+          <t>2026-09-09 12:19</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -806,7 +806,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>dr-hugo-dominguez-malagon</t>
+          <t>dominguez-malagon-patologia</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
+          <t>2018/patologia/2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>2018/patologia/2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2018/patologia/2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>hospital-angeles-lomas</t>
+          <t>hospital-angeles-pedregal</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1468,7 +1468,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1488,35 +1488,35 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>tiroglobulina</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
+          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1536,28 +1536,28 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>tiroglobulina</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024 9:38 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1824,7 +1824,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
+          <t>2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1844,19 +1844,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>biometria-hematica</t>
+          <t>biometria</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>rename</t>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria.pdf') already matches the day-first reading.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023 8:20 AM'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria-hematica.pdf') already matches the day-first reading.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2050,7 +2050,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2022-03-09_labs_quest-usa_tiroideo.pdf</t>
+          <t>2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>tiroglobulina</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2080,12 +2080,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2022/labs/2022-03-09_labs_quest-usa_tiroideo.pdf</t>
+          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2021-06-07_labs_quest-mx_biometria.pdf') — '07/06/2021 9:49 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2021-06-07_labs_quest-mx_biometria.pdf') — '07/06/2021' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -3428,7 +3428,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+          <t>2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>biopsia-tiroides</t>
+          <t>mutacion-braf</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -3458,12 +3458,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3511,7 +3511,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -3614,7 +3614,11 @@
           <t>no_change</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha (encabezado del reporte): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>

</xml_diff>

<commit_message>
chore: update master tracker 2026-09-10 12:14 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-09 12:19</t>
+          <t>2026-09-10 12:14</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -806,7 +806,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>dominguez-malagon-patologia</t>
+          <t>dominguez-malagon</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -831,12 +831,12 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1198,7 +1198,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>hospital-angeles-pedregal</t>
+          <t>hospital-angeles</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-lomas_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1468,7 +1468,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1488,35 +1488,35 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>tiroglobulina</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_general.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
+          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1536,17 +1536,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>tiroglobulina</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2025/labs/2025-10-23_labs_labcorp_tiroglobulina.pdf</t>
+          <t>2025/labs/2025-10-23_labs_labcorp_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1557,7 +1557,7 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://drive.google.com/file/d/15Ufzy5LF4nINVnNLyg9kUHvITUjrp9hO/view</t>
+          <t>https://drive.google.com/file/d/1FuROGZ9o12bFpNUDhxg3X7FiGsWAlMAB/view</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1859,12 +1859,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023 8:20 AM'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria-hematica.pdf') already matches the day-first reading.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria.pdf') already matches the day-first reading.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2022/labs/2022-03-09_labs_quest-usa_tiroideo.pdf</t>
+          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2085,12 +2085,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroideo.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
+          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroglobulina.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2202,7 +2202,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2232,12 +2232,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2021-06-07_labs_quest-mx_biometria.pdf') — '07/06/2021' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2021-06-07_labs_quest-mx_biometria.pdf') — '07/06/2021 9:49 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2750,7 +2750,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2020-06-01_patologia_nucleo-diagnostico_biopsia-tiroides.pdf</t>
+          <t>2020-06-01_patologia_nucleo-diagnostico_citologia-ganglionar.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2770,7 +2770,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>biopsia-tiroides</t>
+          <t>citologia-ganglionar</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2780,15 +2780,19 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_biopsia-tiroides.pdf</t>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-ganglionar.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>no_change</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr"/>
+          <t>rename</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha del reporte (encabezado 'Ciudad de México, a...'): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/19PXsFTn8Hf3QyTUKLZGk5MDFmI978hn4/view</t>
@@ -2902,7 +2906,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2020-06-15_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020-06-15_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2922,7 +2926,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2932,12 +2936,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2020/labs/2020-06-15_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/labs/2020-06-15_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -3453,7 +3457,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -3463,7 +3467,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -3476,7 +3480,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2019-05-15_labs_quest-mx_general-orina.pdf</t>
+          <t>2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3496,7 +3500,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>general-orina</t>
+          <t>general</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -3506,12 +3510,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -3616,7 +3620,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha (encabezado del reporte): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de reporte (encabezado, sin etiqueta explícita de toma de muestra): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">

</xml_diff>

<commit_message>
chore: update master tracker 2026-09-11 12:11 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-10 12:14</t>
+          <t>2026-09-11 12:11</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dominguez-malagon-patologia_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -1198,7 +1198,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>hospital-angeles</t>
+          <t>hospital-angeles-pedregal</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -1223,12 +1223,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1761,7 +1761,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -1824,7 +1824,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>biometria</t>
+          <t>biometria-hematica</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1854,17 +1854,17 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria.pdf') already matches the day-first reading.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023 8:20 AM'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria.pdf') already matches the day-first reading.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1924,7 +1924,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
+          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ultrasonido-cuello</t>
+          <t>ultrasonido-tiroides</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1954,12 +1954,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
@@ -2050,7 +2050,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>2022-03-09_labs_quest-usa_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>tiroglobulina</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -2080,12 +2080,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>2022/labs/2022-03-09_labs_quest-usa_tiroideo.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -2227,7 +2227,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2022/labs/2022-11-22_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2022/labs/2022-11-22_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2237,12 +2237,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022 8:58 AM'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -2702,7 +2702,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>tiroideo</t>
+          <t>perfil-tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2732,12 +2732,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -2750,7 +2750,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2020-06-01_patologia_nucleo-diagnostico_citologia-ganglionar.pdf</t>
+          <t>2020-06-01_patologia_nucleo-diagnostico_citologia-baaf.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2770,17 +2770,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>citologia-ganglionar</t>
+          <t>citologia-baaf</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_biopsia-tiroides.pdf</t>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-ganglionar.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-ganglionar.pdf</t>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-baaf.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha del reporte (encabezado 'Ciudad de México, a...'): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha del reporte (encabezado, Ciudad de México, a...): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -2854,7 +2854,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglionar.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2874,7 +2874,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>biopsia-tiroides</t>
+          <t>biopsia-ganglionar</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2884,12 +2884,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglionar.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -2906,7 +2906,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2020-06-15_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020-06-15_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2926,17 +2926,17 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>perfil-tiroideo</t>
+          <t>tiroideo</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
+          <t>2020/labs/2020-06-15_labs_quest-mx_perfil-tiroideo.pdf</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>2020/labs/2020-06-15_labs_quest-mx_tiroideo.pdf</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2020/labs/2020-06-15_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -3432,7 +3432,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
+          <t>2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3452,7 +3452,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>mutacion-braf</t>
+          <t>biopsia-tiroides</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -3462,12 +3462,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
+          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -3505,7 +3505,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2019/labs/2019-05-15_labs_quest-mx_general-orina.pdf</t>
+          <t>2019/labs/2019-05-15_labs_quest-mx_general.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -3618,11 +3618,7 @@
           <t>no_change</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de reporte (encabezado, sin etiqueta explícita de toma de muestra): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
-        </is>
-      </c>
+      <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>

</xml_diff>

<commit_message>
chore: update master tracker 2026-09-12 11:37 UTC
</commit_message>
<xml_diff>
--- a/tracker/master_tracker.xlsx
+++ b/tracker/master_tracker.xlsx
@@ -465,7 +465,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-11 12:11</t>
+          <t>2026-09-12 11:37</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
@@ -806,7 +806,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2018-12-24_patologia_dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -821,7 +821,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>dominguez-malagon</t>
+          <t>dr-hugo-dominguez-malagon</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -836,12 +836,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2018/patologia/2018-12-24_patologia_dominguez-malagon_biopsia-tiroides.pdf</t>
+          <t>2018/patologia/2018-12-24_patologia_dr-hugo-dominguez-malagon_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>no_change</t>
+          <t>rename</t>
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
@@ -1198,7 +1198,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroideo.pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1218,17 +1218,17 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>ultrasonido-tiroides</t>
+          <t>ultrasonido-tiroideo</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroides.pdf</t>
+          <t>2026/ultrasonidos/2026-04-14_ultrasonidos_hospital-angeles-pedregal_ultrasonido-tiroideo.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024 9:38 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2024-08-10_labs_quest-mx_biometria.pdf') — '10/08/2024' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1761,7 +1761,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -1824,7 +1824,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
+          <t>2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1844,19 +1844,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>biometria-hematica</t>
+          <t>biometria</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>2023/labs/2023-07-12_labs_quest-mx_biometria.pdf</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>2023/labs/2023-07-12_labs_quest-mx_biometria-hematica.pdf</t>
-        </is>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>rename</t>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023 8:20 AM'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria.pdf') already matches the day-first reading.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '12/07/2023'). This is the report date, not a confirmed sample-collection date. That report date was itself ambiguous on its own, but the current filename ('2023-07-12_labs_quest-mx_biometria-hematica.pdf') already matches the day-first reading.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1924,7 +1924,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
+          <t>2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1944,17 +1944,17 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ultrasonido-tiroides</t>
+          <t>ultrasonido-cuello</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-cuello.pdf</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2023/ultrasonidos/2023-07-15_ultrasonidos_clinica-anahuac_ultrasonido-tiroides.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2022/labs/2022-03-09_labs_quest-usa_tiroglobulina.pdf</t>
+          <t>2022/labs/2022-03-09_labs_quest-usa_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -2085,12 +2085,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroglobulina.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
+          <t>date confirmed via existing filename ('2022-03-09_labs_quest-usa_tiroideo.pdf') — '03/09/2022' was ambiguous on its own, but the current name already matches the month-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2242,7 +2242,7 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022 8:58 AM'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha Creación: '22/11/2022'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -2372,7 +2372,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2021-06-07_labs_quest-mx_biometria.pdf') — '07/06/2021 9:49 AM' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2021-06-07_labs_quest-mx_biometria.pdf') — '07/06/2021' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -2495,7 +2495,7 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -2727,7 +2727,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2020/labs/2020-05-25_labs_quest-mx_tiroideo.pdf</t>
+          <t>2020/labs/2020-05-25_labs_quest-mx_perfil-tiroideo.pdf</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2737,7 +2737,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
@@ -2750,7 +2750,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2020-06-01_patologia_nucleo-diagnostico_citologia-baaf.pdf</t>
+          <t>2020-06-01_patologia_nucleo-diagnostico_citologia-ganglio.pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2770,17 +2770,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>citologia-baaf</t>
+          <t>citologia-ganglio</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-ganglionar.pdf</t>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-baaf.pdf</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-baaf.pdf</t>
+          <t>2020/patologia/2020-06-01_patologia_nucleo-diagnostico_citologia-ganglio.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha del reporte (encabezado, Ciudad de México, a...): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha de reporte (encabezado, Ciudad de México, a...): '01 de junio del año 2020'). This is the report date, not a confirmed sample-collection date.</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -2854,7 +2854,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglionar.pdf</t>
+          <t>2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglios-linfaticos.pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2874,17 +2874,17 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>biopsia-ganglionar</t>
+          <t>biopsia-ganglios-linfaticos</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
+          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglionar.pdf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglionar.pdf</t>
+          <t>2020/patologia/2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglios-linfaticos.pdf</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>date confirmed via existing filename ('2020-06-05_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf') — '05-06-2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
+          <t>date confirmed via existing filename ('2020-06-05_patologia_hospital-angeles-pedregal_biopsia-ganglionar.pdf') — '05-06-2020' was ambiguous on its own, but the current name already matches the day-first reading</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -2931,7 +2931,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2020/labs/2020-06-15_labs_quest-mx_perfil-tiroideo.pdf</t>
+          <t>2020/labs/2020-06-15_labs_quest-mx_tiroideo.pdf</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I9" t="inlineStr"/>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_mutacion-braf.pdf</t>
+          <t>2019/patologia/2019-04-29_patologia_hospital-angeles-pedregal_biopsia-tiroides.pdf</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -3467,7 +3467,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>rename</t>
+          <t>no_change</t>
         </is>
       </c>
       <c r="I8" t="inlineStr"/>
@@ -3618,7 +3618,11 @@
           <t>no_change</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>NO COLLECTION DATE ON DOCUMENT — using report/creation date instead (Fecha (encabezado del reporte, sin etiqueta explícita): '21 DE AGOSTO DEL 2019'). This is the report date, not a confirmed sample-collection date.</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
           <t>https://drive.google.com/file/d/1nhYvXwGIEiHvTqmy7bul8-8pVHzfbNaK/view</t>

</xml_diff>